<commit_message>
Cất việc: trạng thái 16/106 vào Excel, và chỗ dừng vào toi-uu/DANG-LAM.md
Hai việc #15 M3-13 và #16 M3-18 đã chốt và gộp main. Không việc nào đang dở.

Excel: sheet mới "Tiến độ 08-10-2026" (16 xong · 0 đang làm · 90 chưa), và cột
Q, T–Y của hai dòng M3-13/M3-18 trong "Danh mục tối ưu". Khối "Lỗi tìm thấy trong
CHÍNH PHÉP ĐO của tôi" thêm bốn dòng — ba trong số đó là chuyện phạm vi phép đo
sai mà vẫn ra một con số hợp lý.

DANG-LAM.md: chỗ dừng là #17 M4-01, và bốn thứ phải đọc trước khi gõ — thêm hai
bài học mới so với bản 07/10: "phá lại thì đỏ N/N" chỉ nói được điều gì khi tập
phép phá không do người đang mong nó đẹp chọn ra, và phạm vi phép đo sai thì ra
một con số HỢP LÝ chứ không ra rỗng.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 07-10-2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -2100,13 +2101,13 @@
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
@@ -3170,6 +3171,1183 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" style="27" min="1" max="1"/>
+    <col width="66" customWidth="1" style="27" min="2" max="2"/>
+    <col width="24" customWidth="1" style="27" min="3" max="3"/>
+    <col width="8" customWidth="1" style="27" min="4" max="4"/>
+    <col width="11" customWidth="1" style="27" min="5" max="5"/>
+    <col width="16" customWidth="1" style="27" min="6" max="6"/>
+    <col width="34" customWidth="1" style="27" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>TIẾN ĐỘ ĐỢT TỐI ƯU TÁC TỬ — chốt ngày 08/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Mỗi dòng 'Xong' đều có: mục DEV-LOG tra lại được · số ca kiểm trước→sau · một con số đo trên dữ liệu thật · phần còn nợ. Cột chi tiết nằm ở sheet “Danh mục tối ưu”, cột T–Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Tổng quan</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Số việc</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Xong (đã gộp vào main, đã đẩy)</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>16 việc đầu của Giai đoạn 1, theo đúng thứ tự # của kế hoạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Đang làm (chưa commit)</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>không việc nào đang dở — M3-13 đã chốt và gộp main sáng 08/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="n">
+        <v>90</v>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>90 việc còn lại trong 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="n">
+        <v>106</v>
+      </c>
+      <c r="C8" s="61" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>Phép đo của cả đợt</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>Trước (06/10)</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Sau (08/10)</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị Python (pytest -q)</t>
+        </is>
+      </c>
+      <c r="B11" s="63" t="inlineStr">
+        <is>
+          <t>1 610</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>1 773</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>+163 ca so với 06/10; không ca cũ nào đỏ ở bất kỳ bước nào</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị giao diện (swift test)</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>không nhiệm vụ nào đụng ui/ — kiểu khối A2.2 dùng “table”, Swift đã dựng được</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="63" t="inlineStr">
+        <is>
+          <t>kiem_tai_lieu.py</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ LỆCH CHẮC CHẮN cả hai lượt. Hôm nay nó bắt đúng chuyện cần bắt: hai công cụ mới làm README lệch số công cụ 127 → 129, và số 'cần đọc lại' nhảy 11 → 15 → về 11 sau khi sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>thu_sch.py (cờ schematic bật)</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>chạy ở M3-03 và M3-04, không tụt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Mục DEV-LOG mới</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330 → DEV-345</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>16 mục, mỗi việc một mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>Cờ tính năng mới</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>1 (schematic)</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>6 cờ mới, TẤT CẢ mặc định TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>Mã lỗi mới</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>E4031 · E4032 · E6012 · E4033</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>E4033 của M3-18 KHÔNG lấy theo kế hoạch: tôi chọn E4031 trước, rồi grep thấy loop.py:1085 đã dùng E4031 cho 'chưa chạy, vì chờ cổng'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>Mảng</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>Ưu tiên</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>DEV-LOG</t>
+        </is>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Ca kiểm</t>
+        </is>
+      </c>
+      <c r="G19" s="59" t="inlineStr">
+        <is>
+          <t>Cờ mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>M1-01</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330</t>
+        </is>
+      </c>
+      <c r="F20" s="63" t="inlineStr">
+        <is>
+          <t>105/309 phiên thật có lịch sử tự mâu thuẫn — 255 chỗ (156 kết quả thứ hai cùng id, 74 message chen giữa, 24 kết quả lạc lượt, 1 lời gọi không kết quả)</t>
+        </is>
+      </c>
+      <c r="G20" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>M1-02</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>DEV-331</t>
+        </is>
+      </c>
+      <c r="F21" s="63" t="inlineStr">
+        <is>
+          <t>lược đồ công cụ thật: 25 869 token/lời gọi (trần tool_schema=4000 chưa dòng mã nào đọc). Cờ bật: 4 475 token, giảm 82,7 %; 73 → 18 công cụ</t>
+        </is>
+      </c>
+      <c r="G21" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>M1-03</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
+        <is>
+          <t>DEV-332</t>
+        </is>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>1 822 lời gọi của tác tử con trong 26 phiên thật, 0 lần qua lớp luật. Toàn công cụ đọc trừ một build.compile — lỗ hổng chưa bị bước vào, không phải được canh</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>M2-01</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>DEV-333</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>kịch bản 3 REQ + 3 phương án + 3 tiêu chí + 3 tệp: sửa MỘT REQ làm 9 hiện vật STALE → còn 3. Phép đo đầu ra 6→2 vì bị hàng rào E4020 chặn, đã sửa kịch bản đo</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="inlineStr">
+        <is>
+          <t>TRUY_VET — TẮT (phần nền chạy cả khi tắt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>M2-02</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E24" s="63" t="inlineStr">
+        <is>
+          <t>DEV-334</t>
+        </is>
+      </c>
+      <c r="F24" s="63" t="inlineStr">
+        <is>
+          <t>63 kho thật: 5/37 REQ có ít nhất một phép đo; 27 chưa có phương án nào nhận; 0 REQ đi hết chuỗi. Cột 'Mã nguồn' trống ở MỌI dự án vì hien_thuc_req vừa mới tồn tại</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="inlineStr">
+        <is>
+          <t>REQ_PHU — TẮT (khối A2.2 trên tab không phụ thuộc cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>M2-03</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E25" s="63" t="inlineStr">
+        <is>
+          <t>DEV-335</t>
+        </is>
+      </c>
+      <c r="F25" s="63" t="inlineStr">
+        <is>
+          <t>37 REQ thật: 25 sạch (67 %), 11 thiếu tiêu chí đo được, 2 có từ mơ hồ. Lần đo đầu ra 3 từ mơ hồ, một là kêu oan ('ít nhất 2 lần' là mức đo được) — đã vá</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="inlineStr">
+        <is>
+          <t>REQ_CHAT_LUONG — TẮT (module yeu_cau.py luôn có)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>M2-06</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="inlineStr">
+        <is>
+          <t>DEV-336</t>
+        </is>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>sổ cái thật: 26 lần đánh dấu 'xong' ngay sau một lần ghi mã, 19 lần (73 %) không có phép kiểm nào đạt ở giữa. Phép đo đầu ở mức dự án ra 0 — đúng nhưng đo sai câu hỏi</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="inlineStr">
+        <is>
+          <t>KE_HOACH_CONG_KIEM — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>M2-08</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="inlineStr">
+        <is>
+          <t>DEV-337</t>
+        </is>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>185 tệp .c thật: 1 758 → 1 786 hàm thấy được (+28 hàm trước đây VÔ HÌNH: 8 ngắt + 20 bị regex tham lam nuốt). 78 hàm nay gắn nhãn 'isr', 70 trong đó vốn đã có trong danh sách</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>DEV-338</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mô hình mạch thật — và lý do đáng hơn con số: 3 kho CÓ Fact v_max thì KHÔNG có mô hình mạch, 5 kho có mạch thì không có Fact ấy; thêm nữa Fact dùng chủ thể chip:X mà ERC không tra tiền tố đó</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E29" s="63" t="inlineStr">
+        <is>
+          <t>DEV-339</t>
+        </is>
+      </c>
+      <c r="F29" s="63" t="inlineStr">
+        <is>
+          <t>8 phát hiện trên 5 mạch thật (6 nguon_khong_cap + 2 net_mot_chan), trong đó net clock I2C nối đúng một chân. SÁU trong tám là 'mô hình chưa khai' chứ không phải 'mạch sai'. robot-canbang: 107 Port lá, KHÔNG Port nào là power_out</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E30" s="63" t="inlineStr">
+        <is>
+          <t>DEV-340</t>
+        </is>
+      </c>
+      <c r="F30" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mạch thật — và đây là con số ĐÚNG (hai lỗi này catastrophic, không bo nào sống tới lúc lưu kho). Đã CẤY hai bộ cấp vào bản sao kho robot-canbang để chứng minh luật sống: nổ đúng 1 blocker trên net +5V thật</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>M3-07</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E31" s="63" t="inlineStr">
+        <is>
+          <t>DEV-341</t>
+        </is>
+      </c>
+      <c r="F31" s="63" t="inlineStr">
+        <is>
+          <t>Fact tới được ERC: 5 → 17 (+12). Ba kho có Fact datasheet thì TOÀN BỘ mang chủ thể chip:, tức trước đó không một Fact nào tới được ERC. Độ phủ 5 mạch thật nay đọc được</t>
+        </is>
+      </c>
+      <c r="G31" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>M3-10</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E32" s="63" t="inlineStr">
+        <is>
+          <t>DEV-342</t>
+        </is>
+      </c>
+      <c r="F32" s="63" t="inlineStr">
+        <is>
+          <t>chi phí đo thật: mạch lớn nhất trong kho 187 nút → ERC 7,6 ms mỗi lần ghi. Trần 2000 nút, vượt thì NÓI RA chứ không im lặng bỏ qua</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="inlineStr">
+        <is>
+          <t>ERC_TU_DONG — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>M3-12</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E33" s="63" t="inlineStr">
+        <is>
+          <t>DEV-343</t>
+        </is>
+      </c>
+      <c r="F33" s="63" t="inlineStr">
+        <is>
+          <t>846 bản ghi mô phỏng thật: regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 (testbench dự án in 'KET QUA: PASS' — nhãn đứng TRƯỚC từ khoá). Nới đúng một chỗ → 846/846 khớp, vẫn bắt đủ bốn ca PASS giả</t>
+        </is>
+      </c>
+      <c r="G33" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="64" t="inlineStr">
+        <is>
+          <t>M3-13</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="inlineStr">
+        <is>
+          <t>DEV-344</t>
+        </is>
+      </c>
+      <c r="F34" s="64" t="inlineStr">
+        <is>
+          <t>testbench Verilog THẬT của bài 3: tb_pcpi_dot4 1/1, tb_pcpi_mac 1/1, tb_pcpi_vmini không đo được (tb gọi bản bram HAI CỔNG đã bị bỏ 02/10) — mẫu số là TỆP, không phải phép phá</t>
+        </is>
+      </c>
+      <c r="G34" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>M3-18</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="inlineStr">
+        <is>
+          <t>DEV-345</t>
+        </is>
+      </c>
+      <c r="F35" s="64" t="inlineStr">
+        <is>
+          <t>6 cặp (mạng cổng, .cst) thật → 1 chỗ CHẶN: blinky của riscv-tn20k-b dựng bitstream 4,6 MB với chân đồng hồ do nextpnr tự chọn (rơi đúng chân 4 — bằng may). Cả 7 tệp .cst thật đọc hết, 0 lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="G35" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="59" t="inlineStr">
+        <is>
+          <t>Việc còn MỞ (ngoài 90 việc chưa làm)</t>
+        </is>
+      </c>
+      <c r="B37" s="59" t="inlineStr">
+        <is>
+          <t>Vì sao còn mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="63" t="inlineStr">
+        <is>
+          <t>Sáu cờ mới đều còn TẮT</t>
+        </is>
+      </c>
+      <c r="B38" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU · TRUY_VET · REQ_PHU · REQ_CHAT_LUONG · KE_HOACH_CONG_KIEM · ERC_TU_DONG. Cả sáu đổi thứ Agent nhìn thấy hoặc đọc mỗi lượt, nên chỉ bộ 76 ca chạy HAI chế độ mới nói được chúng làm Agent khá hơn hay tệ hơn — bộ ấy tốn tiền mô hình nên chưa chạy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="63" t="inlineStr">
+        <is>
+          <t>kiem_cap_goi_tra() chưa thành hàng rào</t>
+        </is>
+      </c>
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t>Soát được mọi phiên đã lưu, nhưng chưa hook nào gọi nó tự động — bắt được chuyện cũ, chưa chặn được chuyện mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="63" t="inlineStr">
+        <is>
+          <t>Luật ERC quá áp chưa nổ trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="B40" s="63" t="inlineStr">
+        <is>
+          <t>Đường dẫn đã thông ở M3-07, nhưng ba kho có Fact điện áp thì không có mô hình mạch, và ngược lại. Phải chờ một dự án có cả hai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="63" t="inlineStr">
+        <is>
+          <t>Cột “Mã nguồn” của ma trận truy vết trống ở mọi dự án</t>
+        </is>
+      </c>
+      <c r="B41" s="63" t="inlineStr">
+        <is>
+          <t>Nó đọc hien_thuc_req — trường vừa mới tồn tại, chưa tệp nào trên đĩa từng khai. Nên “chưa hiện thực” ở đó nghĩa là “chưa ai KHAI”, không phải “chưa ai viết”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="63" t="inlineStr">
+        <is>
+          <t>Lỗi _go_dau trong src/eide/tools/design.py</t>
+        </is>
+      </c>
+      <c r="B42" s="63" t="inlineStr">
+        <is>
+          <t>Viết .replace('d','d') nên 'ổn định' và 'ON DINH' không khớp nhau. Hàm ấy đang dùng cho một phép kiểm an toàn (người có thật sự chọn không). Tìm thấy ở M2-03, CHƯA sửa vì ngoài phạm vi — cần bộ ca kiểm riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="63" t="inlineStr">
+        <is>
+          <t>subagent req-critic (bước 4 của M2-03)</t>
+        </is>
+      </c>
+      <c r="B43" s="63" t="inlineStr">
+        <is>
+          <t>Kế hoạch ghi “tuỳ chọn, gộp M2-13”. Chưa làm, đúng theo kế hoạch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="63" t="inlineStr">
+        <is>
+          <t>Hai luật kiểm chân FPGA chưa có dữ liệu để nổ</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="inlineStr">
+        <is>
+          <t>chan_lech_kit và io_type_lech_bank cần Fact chân kit. Không kho nào trong repo có Fact pin:tangnano20k.* hay khoá vccio — nên hôm nay chỉ 3 trong 5 luật của M3-18 kết luận được gì trên dữ liệu thật. Cùng hình dạng với luật ERC quá áp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="63" t="inlineStr">
+        <is>
+          <t>Một bitstream cũ đã dựng với chân đồng hồ tự chọn</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="inlineStr">
+        <is>
+          <t>blinky của du-lieu/riscv-tn20k-b — xem DEV-345 và README §8. Không sửa hiện vật cũ: đó là dữ liệu của những lượt đo đã chốt. Từ nay phép kiểm chặn trước nextpnr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="63" t="inlineStr">
+        <is>
+          <t>Hai công cụ mới nhất chưa lượt Agent nào GỌI</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="inlineStr">
+        <is>
+          <t>hdl.sensitivity và hdl.constraints_check: mã của cả hai đã chạy trên hiện vật thật, nhưng đó là tôi gọi hàm, không phải tác tử gọi công cụ. README §8 đếm cả hai vào phần chưa dùng thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="59" t="inlineStr">
+        <is>
+          <t>Lỗi tìm thấy trong CHÍNH PHÉP ĐO của tôi</t>
+        </is>
+      </c>
+      <c r="B48" s="59" t="inlineStr">
+        <is>
+          <t>Lộ ra ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="63" t="inlineStr">
+        <is>
+          <t>Kịch bản đo bị hàng rào của sản phẩm chặn (ghi tệp chưa đọc, E4020) và trả về một con số hợp lý thay vì nổ — 6→2 trông đẹp y như 9→3 đúng</t>
+        </is>
+      </c>
+      <c r="B49" s="63" t="inlineStr">
+        <is>
+          <t>M2-01 · DEV-333</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm dựng trên điều tôi tự nhớ sai: “thiết” bỏ dấu KHÔNG chứa “it”; chỗ va thật là bit/unit/init/exit</t>
+        </is>
+      </c>
+      <c r="B50" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá dài ĐÚNG BẰNG mã gốc (0.6 → 0.0) nên __pycache__ cũ còn hiệu lực — phép đo chạy mã khác với mã trong tệp</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="63" t="inlineStr">
+        <is>
+          <t>Phép đo trả lời ĐÚNG một câu hỏi KHÁC: đếm ở mức dự án ra 0 chỗ cần chặn; câu phải hỏi là “lần ghi NÀY đã được kiểm chưa” → 19/26</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="inlineStr">
+        <is>
+          <t>M2-06 · DEV-336</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm RỖNG: dàn dựng không có net đất nào, nên nó xanh cả khi tôi bỏ hẳn phép bỏ qua net đất</t>
+        </is>
+      </c>
+      <c r="B53" s="63" t="inlineStr">
+        <is>
+          <t>M3-01 · DEV-338</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="63" t="inlineStr">
+        <is>
+          <t>Hai phép phá chỉ ra THIẾT KẾ sai, không chỉ ca kiểm yếu (miễn net đất quá rộng; nhánh iout_max chưa ca nào chạm tới)</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="inlineStr">
+        <is>
+          <t>M3-03 · DEV-339</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá của tôi cũng SAI, và ca âm xanh vì lý do khác — hai cái sai che nhau</t>
+        </is>
+      </c>
+      <c r="B55" s="63" t="inlineStr">
+        <is>
+          <t>M3-07 · DEV-341</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm đo chính câu lệnh của mình (đặt bộ đếm = 3 rồi khẳng định nó khác rỗng, trong khi thực tế nó rỗng)</t>
+        </is>
+      </c>
+      <c r="B56" s="63" t="inlineStr">
+        <is>
+          <t>M3-10 · DEV-342</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="63" t="inlineStr">
+        <is>
+          <t>Regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 bản ghi thật; và ba ca kiểm xanh vì lý do sai (tệp giả dùng $4 thay $3; “FAILED” chứa “FAIL”)</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="inlineStr">
+        <is>
+          <t>M3-12 · DEV-343</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="63" t="inlineStr">
+        <is>
+          <t>"Phá lại thì đỏ 6/6" sai về TẬP, không sai về số: sáu phép phá ấy chọn đúng sáu chỗ đã có ca canh. Phá bằng tập rộng hơn ra 7/9.</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="inlineStr">
+        <is>
+          <t>M3-13 · DEV-344</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="63" t="inlineStr">
+        <is>
+          <t>409 'blocker' gần như toàn bộ từ một cặp vô nghĩa (mạng cổng của lõi CPU tổng hợp riêng, không bao giờ đem đặt-đi dây). Con số thật là 1.</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="63" t="inlineStr">
+        <is>
+          <t>Phép quét tệp .cst thật chỉ thu 4 trong 7 tệp mà ca kiểm vẫn xanh — câu 'mọi tệp .cst thật đều đọc được' nói về phần phép quét chạm tới.</t>
+        </is>
+      </c>
+      <c r="B60" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="63" t="inlineStr">
+        <is>
+          <t>Một ca kiểm và một phép phá nhắm hai NHÁNH khác nhau, nên ca mới xanh mà phép phá vẫn LỌT. Mất một lượt mới thấy.</t>
+        </is>
+      </c>
+      <c r="B61" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="63" t="n"/>
+      <c r="B62" s="63" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8473,7 +9651,7 @@
       </c>
       <c r="Q58" s="51" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="R58" s="47" t="inlineStr">
@@ -8484,22 +9662,22 @@
       <c r="S58" s="47" t="n"/>
       <c r="T58" s="52" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="U58" s="52" t="inlineStr">
         <is>
-          <t>chưa ghi</t>
+          <t>DEV-344</t>
         </is>
       </c>
       <c r="V58" s="52" t="inlineStr">
         <is>
-          <t>chưa chạy toàn bộ</t>
+          <t>1732 → 1744 (+12)</t>
         </is>
       </c>
       <c r="W58" s="52" t="inlineStr">
         <is>
-          <t>testbench Verilog THẬT của bài 3 (lõi RISC-V): pcpi_dot4 bắt 1/1, pcpi_mac bắt 1/1 (phép phá 'đảo điều kiện if' làm bộ kiểm đỏ); pcpi_vmini CHƯA đo được — tb cần thêm mô-đun ram ngoài phần nó tự include</t>
+          <t>testbench Verilog THẬT của bài 3 (lõi RISC-V), đo lại qua chính đường mã của công cụ trên một BẢN SAO của docs/riscv-tn20k: tb_pcpi_dot4 1/1 (đảo if, 3 chỗ → bộ kiểm ĐỎ), tb_pcpi_mac 1/1 (đảo if, 2 chỗ). tb_pcpi_vmini KHÔNG đo được — và cổng 'bộ kiểm phải XANH trước khi đo' chặn đúng: tb tạo thực thể bram với 5 cổng b_* của bản HAI CỔNG, mà rtl/bram.v đã về một cổng ngày 02/10/2026. Testbench nấc 3c không dịch nổi từ hôm ấy, trong khi bai3/NGOAI-PHAM-VI.md vẫn ghi 'độ nhạy 7/7'.</t>
         </is>
       </c>
       <c r="X58" s="52" t="inlineStr">
@@ -8509,7 +9687,7 @@
       </c>
       <c r="Y58" s="52" t="inlineStr">
         <is>
-          <t>ĐANG DỞ trên nhánh toi-uu/M3-13, CHƯA commit: đã có PHEP_VERILOG, do_do_nhay_hdl(), công cụ hdl.sensitivity, nhãn do_bang='tu_khai' và dòng 'tự khai' trên khối A8.0; 6 phép phá đều đỏ; CÒN LẠI: chạy pytest toàn bộ, kiem_tai_lieu, ghi DEV-LOG, commit</t>
+          <t>MẪU SỐ LÀ TỆP, không phải phép phá: do_do_nhay break ngay khi một phép làm bộ kiểm đỏ, nên '1/1' nghĩa là 1 trong 1 TỆP RTL — không so được với '7/7 phép' của bản đo tay. Nhãn A8.0 và note_vi đã sửa theo do_bang. · 'phá lại thì đỏ 6/6' của bản WIP là 7/9 khi phá bằng tập rộng hơn: hai chỗ LỌT là bang=PHEP_VERILOG và cổng 'bộ kiểm phải XANH'. Bù TC-07/08/09, phá lại 9/9. · Công cụ thứ 128 này CHƯA lượt Agent nào gọi.</t>
         </is>
       </c>
     </row>
@@ -8935,11 +10113,45 @@
       <c r="P63" s="47" t="n"/>
       <c r="Q63" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R63" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R63" s="47" t="inlineStr">
+        <is>
+          <t>Agent (Claude Opus 5)</t>
+        </is>
+      </c>
       <c r="S63" s="47" t="n"/>
+      <c r="T63" s="26" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="U63" s="26" t="inlineStr">
+        <is>
+          <t>DEV-345</t>
+        </is>
+      </c>
+      <c r="V63" s="26" t="inlineStr">
+        <is>
+          <t>1744 → 1773 (+29)</t>
+        </is>
+      </c>
+      <c r="W63" s="26" t="inlineStr">
+        <is>
+          <t>6 cặp (mạng cổng, .cst) THẬT trong du-lieu/ → 1 chỗ CHẶN, và nó đã đi tới bitstream: blinky.v của riscv-tn20k-b khai cổng sys_clk, .cst chỉ khai clk_27m, không tệp .cst nào trong repo có IO_LOC cho sys_clk. nextpnr vẫn chạy; blinky.fs 4,6 MB dựng ra 01/10/2026. sys_clk rơi vào X0Y6/IOBA — cùng ô mà clk_27m (chân 4, CÓ IO_LOC) của soc_top được gán, nên bitstream ấy có thể đã chạy đúng: bằng may, không bằng ràng buộc. Và cả 7 tệp .cst thật trong repo đọc hết, 0 dòng sai cú pháp.</t>
+        </is>
+      </c>
+      <c r="X63" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+      <c r="Y63" s="26" t="inlineStr">
+        <is>
+          <t>409 'blocker' của lượt chạy đầu gần như toàn bộ từ picorv32.json — mạng cổng của lõi CPU tổng hợp riêng để đếm ô, không bao giờ đem đặt-đi dây. Con số thật là 1. · Phép quét tệp .cst thật bản đầu chỉ thu 4/7 tệp mà ca kiểm vẫn xanh. · Hai luật chan_lech_kit và io_type_lech_bank CHƯA có dữ liệu để nổ: không kho nào trong repo có Fact pin:tangnano20k.* hay khoá vccio — nên cst.kiem trả thêm chua_co_fact_chan_kit mức info. · Mã lỗi E4033, không E4031 (loop.py đã dùng cho 'chưa chạy, vì chờ cổng'). · Chưa lượt Agent nào gọi.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="68.25" customHeight="1" s="27">
       <c r="A64" s="46" t="inlineStr">
@@ -13022,7 +14234,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13863,7 +15075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14318,7 +15530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Cất việc: trạng thái 17/106 vào Excel, và chỗ dừng vào toi-uu/DANG-LAM.md
Việc #17 M4-01 đã chốt và gộp main. Không việc nào đang dở.

Excel: sheet mới "Tiến độ 08-10-2026 (chiều)" (17 xong · 0 đang làm · 89 chưa), và
cột Q, T–Y của dòng M4-01 trong "Danh mục tối ưu". Khối "Lỗi tìm thấy trong CHÍNH
PHÉP ĐO của tôi" thêm hai dòng: ca kiểm xanh nhờ một DÒNG KHÁC, và một phép phá
vô hiệu báo LỌT oan.

DANG-LAM.md: chỗ dừng là #18 M4-02, và "năm thứ phải đọc trước khi gõ" — thêm bài
học mới: soi đúng một dòng chứ đừng soi cả khối, và kiểm lại chính phép phá của
mình. Thêm một việc còn mở: chưa kho nào có tiêu chí unit test, nên test.run ở mọi
dự án đang có vẫn đi đường tự khai.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -10,13 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 07-10-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026 (chiều)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -2098,17 +2099,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B53:G53"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -4348,6 +4349,1241 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" style="27" min="1" max="1"/>
+    <col width="66" customWidth="1" style="27" min="2" max="2"/>
+    <col width="24" customWidth="1" style="27" min="3" max="3"/>
+    <col width="8" customWidth="1" style="27" min="4" max="4"/>
+    <col width="11" customWidth="1" style="27" min="5" max="5"/>
+    <col width="16" customWidth="1" style="27" min="6" max="6"/>
+    <col width="34" customWidth="1" style="27" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>TIẾN ĐỘ ĐỢT TỐI ƯU TÁC TỬ — chốt chiều 08/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Mỗi dòng 'Xong' đều có: mục DEV-LOG tra lại được · số ca kiểm trước→sau · một con số đo trên dữ liệu thật · phần còn nợ. Cột chi tiết nằm ở sheet “Danh mục tối ưu”, cột T–Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Tổng quan</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Số việc</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Xong (đã gộp vào main, đã đẩy)</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="n">
+        <v>17</v>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>17 việc đầu của Giai đoạn 1, theo đúng thứ tự # của kế hoạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Đang làm (chưa commit)</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>không việc nào đang dở</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="n">
+        <v>89</v>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>89 việc còn lại trong 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="n">
+        <v>106</v>
+      </c>
+      <c r="C8" s="61" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>Phép đo của cả đợt</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>Trước (06/10)</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Sau (08/10)</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị Python (pytest -q)</t>
+        </is>
+      </c>
+      <c r="B11" s="63" t="inlineStr">
+        <is>
+          <t>1 610</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>1 791</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>+181 ca so với 06/10; không ca cũ nào đỏ ở bất kỳ bước nào</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị giao diện (swift test)</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>không nhiệm vụ nào đụng ui/ — kiểu khối A2.2 dùng “table”, Swift đã dựng được</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="63" t="inlineStr">
+        <is>
+          <t>kiem_tai_lieu.py</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ LỆCH CHẮC CHẮN cả hai lượt. Hôm nay nó bắt đúng chuyện cần bắt: hai công cụ mới làm README lệch số công cụ 127 → 129, và số 'cần đọc lại' nhảy 11 → 15 → về 11 sau khi sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>thu_sch.py (cờ schematic bật)</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>chạy ở M3-03 và M3-04, không tụt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Mục DEV-LOG mới</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330 → DEV-346</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>17 mục, mỗi việc một mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>Cờ tính năng mới</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>1 (schematic)</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>6 cờ mới, TẤT CẢ mặc định TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>Mã lỗi mới</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>E4031 · E4032 · E6012 · E4033 · E4024</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>E4033 (M3-18) và E4024 (M4-01). M4-01 còn DÙNG LẠI E4008/E4009/E4023 của sim.run — cùng một chuyện thì cùng một mã, một mã mới cho cùng một chuyện là bắt người đọc học hai lần</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>Mảng</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>Ưu tiên</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>DEV-LOG</t>
+        </is>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Ca kiểm</t>
+        </is>
+      </c>
+      <c r="G19" s="59" t="inlineStr">
+        <is>
+          <t>Cờ mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>M1-01</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330</t>
+        </is>
+      </c>
+      <c r="F20" s="63" t="inlineStr">
+        <is>
+          <t>105/309 phiên thật có lịch sử tự mâu thuẫn — 255 chỗ (156 kết quả thứ hai cùng id, 74 message chen giữa, 24 kết quả lạc lượt, 1 lời gọi không kết quả)</t>
+        </is>
+      </c>
+      <c r="G20" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>M1-02</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>DEV-331</t>
+        </is>
+      </c>
+      <c r="F21" s="63" t="inlineStr">
+        <is>
+          <t>lược đồ công cụ thật: 25 869 token/lời gọi (trần tool_schema=4000 chưa dòng mã nào đọc). Cờ bật: 4 475 token, giảm 82,7 %; 73 → 18 công cụ</t>
+        </is>
+      </c>
+      <c r="G21" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>M1-03</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
+        <is>
+          <t>DEV-332</t>
+        </is>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>1 822 lời gọi của tác tử con trong 26 phiên thật, 0 lần qua lớp luật. Toàn công cụ đọc trừ một build.compile — lỗ hổng chưa bị bước vào, không phải được canh</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>M2-01</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>DEV-333</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>kịch bản 3 REQ + 3 phương án + 3 tiêu chí + 3 tệp: sửa MỘT REQ làm 9 hiện vật STALE → còn 3. Phép đo đầu ra 6→2 vì bị hàng rào E4020 chặn, đã sửa kịch bản đo</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="inlineStr">
+        <is>
+          <t>TRUY_VET — TẮT (phần nền chạy cả khi tắt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>M2-02</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E24" s="63" t="inlineStr">
+        <is>
+          <t>DEV-334</t>
+        </is>
+      </c>
+      <c r="F24" s="63" t="inlineStr">
+        <is>
+          <t>63 kho thật: 5/37 REQ có ít nhất một phép đo; 27 chưa có phương án nào nhận; 0 REQ đi hết chuỗi. Cột 'Mã nguồn' trống ở MỌI dự án vì hien_thuc_req vừa mới tồn tại</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="inlineStr">
+        <is>
+          <t>REQ_PHU — TẮT (khối A2.2 trên tab không phụ thuộc cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>M2-03</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E25" s="63" t="inlineStr">
+        <is>
+          <t>DEV-335</t>
+        </is>
+      </c>
+      <c r="F25" s="63" t="inlineStr">
+        <is>
+          <t>37 REQ thật: 25 sạch (67 %), 11 thiếu tiêu chí đo được, 2 có từ mơ hồ. Lần đo đầu ra 3 từ mơ hồ, một là kêu oan ('ít nhất 2 lần' là mức đo được) — đã vá</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="inlineStr">
+        <is>
+          <t>REQ_CHAT_LUONG — TẮT (module yeu_cau.py luôn có)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>M2-06</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="inlineStr">
+        <is>
+          <t>DEV-336</t>
+        </is>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>sổ cái thật: 26 lần đánh dấu 'xong' ngay sau một lần ghi mã, 19 lần (73 %) không có phép kiểm nào đạt ở giữa. Phép đo đầu ở mức dự án ra 0 — đúng nhưng đo sai câu hỏi</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="inlineStr">
+        <is>
+          <t>KE_HOACH_CONG_KIEM — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>M2-08</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="inlineStr">
+        <is>
+          <t>DEV-337</t>
+        </is>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>185 tệp .c thật: 1 758 → 1 786 hàm thấy được (+28 hàm trước đây VÔ HÌNH: 8 ngắt + 20 bị regex tham lam nuốt). 78 hàm nay gắn nhãn 'isr', 70 trong đó vốn đã có trong danh sách</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>DEV-338</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mô hình mạch thật — và lý do đáng hơn con số: 3 kho CÓ Fact v_max thì KHÔNG có mô hình mạch, 5 kho có mạch thì không có Fact ấy; thêm nữa Fact dùng chủ thể chip:X mà ERC không tra tiền tố đó</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E29" s="63" t="inlineStr">
+        <is>
+          <t>DEV-339</t>
+        </is>
+      </c>
+      <c r="F29" s="63" t="inlineStr">
+        <is>
+          <t>8 phát hiện trên 5 mạch thật (6 nguon_khong_cap + 2 net_mot_chan), trong đó net clock I2C nối đúng một chân. SÁU trong tám là 'mô hình chưa khai' chứ không phải 'mạch sai'. robot-canbang: 107 Port lá, KHÔNG Port nào là power_out</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E30" s="63" t="inlineStr">
+        <is>
+          <t>DEV-340</t>
+        </is>
+      </c>
+      <c r="F30" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mạch thật — và đây là con số ĐÚNG (hai lỗi này catastrophic, không bo nào sống tới lúc lưu kho). Đã CẤY hai bộ cấp vào bản sao kho robot-canbang để chứng minh luật sống: nổ đúng 1 blocker trên net +5V thật</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>M3-07</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E31" s="63" t="inlineStr">
+        <is>
+          <t>DEV-341</t>
+        </is>
+      </c>
+      <c r="F31" s="63" t="inlineStr">
+        <is>
+          <t>Fact tới được ERC: 5 → 17 (+12). Ba kho có Fact datasheet thì TOÀN BỘ mang chủ thể chip:, tức trước đó không một Fact nào tới được ERC. Độ phủ 5 mạch thật nay đọc được</t>
+        </is>
+      </c>
+      <c r="G31" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>M3-10</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E32" s="63" t="inlineStr">
+        <is>
+          <t>DEV-342</t>
+        </is>
+      </c>
+      <c r="F32" s="63" t="inlineStr">
+        <is>
+          <t>chi phí đo thật: mạch lớn nhất trong kho 187 nút → ERC 7,6 ms mỗi lần ghi. Trần 2000 nút, vượt thì NÓI RA chứ không im lặng bỏ qua</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="inlineStr">
+        <is>
+          <t>ERC_TU_DONG — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>M3-12</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E33" s="63" t="inlineStr">
+        <is>
+          <t>DEV-343</t>
+        </is>
+      </c>
+      <c r="F33" s="63" t="inlineStr">
+        <is>
+          <t>846 bản ghi mô phỏng thật: regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 (testbench dự án in 'KET QUA: PASS' — nhãn đứng TRƯỚC từ khoá). Nới đúng một chỗ → 846/846 khớp, vẫn bắt đủ bốn ca PASS giả</t>
+        </is>
+      </c>
+      <c r="G33" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="64" t="inlineStr">
+        <is>
+          <t>M3-13</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="inlineStr">
+        <is>
+          <t>DEV-344</t>
+        </is>
+      </c>
+      <c r="F34" s="64" t="inlineStr">
+        <is>
+          <t>testbench Verilog THẬT của bài 3: tb_pcpi_dot4 1/1, tb_pcpi_mac 1/1, tb_pcpi_vmini không đo được (tb gọi bản bram HAI CỔNG đã bị bỏ 02/10) — mẫu số là TỆP, không phải phép phá</t>
+        </is>
+      </c>
+      <c r="G34" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>M3-18</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="inlineStr">
+        <is>
+          <t>DEV-345</t>
+        </is>
+      </c>
+      <c r="F35" s="64" t="inlineStr">
+        <is>
+          <t>6 cặp (mạng cổng, .cst) thật → 1 chỗ CHẶN: blinky của riscv-tn20k-b dựng bitstream 4,6 MB với chân đồng hồ do nextpnr tự chọn (rơi đúng chân 4 — bằng may). Cả 7 tệp .cst thật đọc hết, 0 lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="G35" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B36" s="64" t="inlineStr">
+        <is>
+          <t>M4-01</t>
+        </is>
+      </c>
+      <c r="C36" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D36" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E36" s="64" t="inlineStr">
+        <is>
+          <t>DEV-346</t>
+        </is>
+      </c>
+      <c r="F36" s="64" t="inlineStr">
+        <is>
+          <t>18 ca chạy trình biên dịch C thật: tệp test in số đo {"T1":300} với ngưỡng &lt;=255 → EIDE phán 1 ca HỎNG. Chưa kho cũ nào có tiêu chí unit test để đo lại trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="G36" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="59" t="inlineStr">
+        <is>
+          <t>Việc còn MỞ (ngoài 89 việc chưa làm)</t>
+        </is>
+      </c>
+      <c r="B38" s="59" t="inlineStr">
+        <is>
+          <t>Vì sao còn mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="63" t="inlineStr">
+        <is>
+          <t>Sáu cờ mới đều còn TẮT</t>
+        </is>
+      </c>
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU · TRUY_VET · REQ_PHU · REQ_CHAT_LUONG · KE_HOACH_CONG_KIEM · ERC_TU_DONG. Cả sáu đổi thứ Agent nhìn thấy hoặc đọc mỗi lượt, nên chỉ bộ 76 ca chạy HAI chế độ mới nói được chúng làm Agent khá hơn hay tệ hơn — bộ ấy tốn tiền mô hình nên chưa chạy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="63" t="inlineStr">
+        <is>
+          <t>kiem_cap_goi_tra() chưa thành hàng rào</t>
+        </is>
+      </c>
+      <c r="B40" s="63" t="inlineStr">
+        <is>
+          <t>Soát được mọi phiên đã lưu, nhưng chưa hook nào gọi nó tự động — bắt được chuyện cũ, chưa chặn được chuyện mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="63" t="inlineStr">
+        <is>
+          <t>Luật ERC quá áp chưa nổ trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="B41" s="63" t="inlineStr">
+        <is>
+          <t>Đường dẫn đã thông ở M3-07, nhưng ba kho có Fact điện áp thì không có mô hình mạch, và ngược lại. Phải chờ một dự án có cả hai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="63" t="inlineStr">
+        <is>
+          <t>Cột “Mã nguồn” của ma trận truy vết trống ở mọi dự án</t>
+        </is>
+      </c>
+      <c r="B42" s="63" t="inlineStr">
+        <is>
+          <t>Nó đọc hien_thuc_req — trường vừa mới tồn tại, chưa tệp nào trên đĩa từng khai. Nên “chưa hiện thực” ở đó nghĩa là “chưa ai KHAI”, không phải “chưa ai viết”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="63" t="inlineStr">
+        <is>
+          <t>Lỗi _go_dau trong src/eide/tools/design.py</t>
+        </is>
+      </c>
+      <c r="B43" s="63" t="inlineStr">
+        <is>
+          <t>Viết .replace('d','d') nên 'ổn định' và 'ON DINH' không khớp nhau. Hàm ấy đang dùng cho một phép kiểm an toàn (người có thật sự chọn không). Tìm thấy ở M2-03, CHƯA sửa vì ngoài phạm vi — cần bộ ca kiểm riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="63" t="inlineStr">
+        <is>
+          <t>subagent req-critic (bước 4 của M2-03)</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="inlineStr">
+        <is>
+          <t>Kế hoạch ghi “tuỳ chọn, gộp M2-13”. Chưa làm, đúng theo kế hoạch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="63" t="inlineStr">
+        <is>
+          <t>Hai luật kiểm chân FPGA chưa có dữ liệu để nổ</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="inlineStr">
+        <is>
+          <t>chan_lech_kit và io_type_lech_bank cần Fact chân kit. Không kho nào trong repo có Fact pin:tangnano20k.* hay khoá vccio — nên hôm nay chỉ 3 trong 5 luật của M3-18 kết luận được gì trên dữ liệu thật. Cùng hình dạng với luật ERC quá áp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="63" t="inlineStr">
+        <is>
+          <t>Một bitstream cũ đã dựng với chân đồng hồ tự chọn</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="inlineStr">
+        <is>
+          <t>blinky của du-lieu/riscv-tn20k-b — xem DEV-345 và README §8. Không sửa hiện vật cũ: đó là dữ liệu của những lượt đo đã chốt. Từ nay phép kiểm chặn trước nextpnr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="63" t="inlineStr">
+        <is>
+          <t>Ba công cụ mới nhất chưa lượt Agent nào GỌI</t>
+        </is>
+      </c>
+      <c r="B47" s="63" t="inlineStr">
+        <is>
+          <t>hdl.sensitivity · hdl.constraints_check · test.criteria. Mã của cả ba đã chạy trên hiện vật thật, nhưng đó là tôi gọi hàm, không phải tác tử gọi công cụ. README §8 đếm cả ba vào phần chưa dùng thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="59" t="inlineStr">
+        <is>
+          <t>Lỗi tìm thấy trong CHÍNH PHÉP ĐO của tôi</t>
+        </is>
+      </c>
+      <c r="B49" s="59" t="inlineStr">
+        <is>
+          <t>Lộ ra ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="63" t="inlineStr">
+        <is>
+          <t>Kịch bản đo bị hàng rào của sản phẩm chặn (ghi tệp chưa đọc, E4020) và trả về một con số hợp lý thay vì nổ — 6→2 trông đẹp y như 9→3 đúng</t>
+        </is>
+      </c>
+      <c r="B50" s="63" t="inlineStr">
+        <is>
+          <t>M2-01 · DEV-333</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm dựng trên điều tôi tự nhớ sai: “thiết” bỏ dấu KHÔNG chứa “it”; chỗ va thật là bit/unit/init/exit</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá dài ĐÚNG BẰNG mã gốc (0.6 → 0.0) nên __pycache__ cũ còn hiệu lực — phép đo chạy mã khác với mã trong tệp</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="63" t="inlineStr">
+        <is>
+          <t>Phép đo trả lời ĐÚNG một câu hỏi KHÁC: đếm ở mức dự án ra 0 chỗ cần chặn; câu phải hỏi là “lần ghi NÀY đã được kiểm chưa” → 19/26</t>
+        </is>
+      </c>
+      <c r="B53" s="63" t="inlineStr">
+        <is>
+          <t>M2-06 · DEV-336</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm RỖNG: dàn dựng không có net đất nào, nên nó xanh cả khi tôi bỏ hẳn phép bỏ qua net đất</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="inlineStr">
+        <is>
+          <t>M3-01 · DEV-338</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="63" t="inlineStr">
+        <is>
+          <t>Hai phép phá chỉ ra THIẾT KẾ sai, không chỉ ca kiểm yếu (miễn net đất quá rộng; nhánh iout_max chưa ca nào chạm tới)</t>
+        </is>
+      </c>
+      <c r="B55" s="63" t="inlineStr">
+        <is>
+          <t>M3-03 · DEV-339</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá của tôi cũng SAI, và ca âm xanh vì lý do khác — hai cái sai che nhau</t>
+        </is>
+      </c>
+      <c r="B56" s="63" t="inlineStr">
+        <is>
+          <t>M3-07 · DEV-341</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm đo chính câu lệnh của mình (đặt bộ đếm = 3 rồi khẳng định nó khác rỗng, trong khi thực tế nó rỗng)</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="inlineStr">
+        <is>
+          <t>M3-10 · DEV-342</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="63" t="inlineStr">
+        <is>
+          <t>Regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 bản ghi thật; và ba ca kiểm xanh vì lý do sai (tệp giả dùng $4 thay $3; “FAILED” chứa “FAIL”)</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="inlineStr">
+        <is>
+          <t>M3-12 · DEV-343</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="63" t="inlineStr">
+        <is>
+          <t>"Phá lại thì đỏ 6/6" sai về TẬP, không sai về số: sáu phép phá ấy chọn đúng sáu chỗ đã có ca canh. Phá bằng tập rộng hơn ra 7/9.</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="inlineStr">
+        <is>
+          <t>M3-13 · DEV-344</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="63" t="inlineStr">
+        <is>
+          <t>409 'blocker' gần như toàn bộ từ một cặp vô nghĩa (mạng cổng của lõi CPU tổng hợp riêng, không bao giờ đem đặt-đi dây). Con số thật là 1.</t>
+        </is>
+      </c>
+      <c r="B60" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="63" t="inlineStr">
+        <is>
+          <t>Phép quét tệp .cst thật chỉ thu 4 trong 7 tệp mà ca kiểm vẫn xanh — câu 'mọi tệp .cst thật đều đọc được' nói về phần phép quét chạm tới.</t>
+        </is>
+      </c>
+      <c r="B61" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="63" t="inlineStr">
+        <is>
+          <t>Một ca kiểm và một phép phá nhắm hai NHÁNH khác nhau, nên ca mới xanh mà phép phá vẫn LỌT. Mất một lượt mới thấy.</t>
+        </is>
+      </c>
+      <c r="B62" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm xanh nhờ một DÒNG KHÁC: kiểm `"TỰ KHAI" in str(kh)` cả khối nên vẫn xanh khi phá chữ ấy ở dòng Kết luận — summary cũng chứa nó. Phép phá bắt được, ca kiểm thì không.</t>
+        </is>
+      </c>
+      <c r="B63" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="63" t="inlineStr">
+        <is>
+          <t>Một phép phá VÔ HIỆU: `them = [] or [[…]]` không đổi hành vi, nên nó báo LỌT oan và suýt làm tôi viết ca kiểm cho một chỗ vốn đã được canh.</t>
+        </is>
+      </c>
+      <c r="B64" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10575,11 +11811,45 @@
       <c r="P68" s="47" t="n"/>
       <c r="Q68" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R68" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R68" s="47" t="inlineStr">
+        <is>
+          <t>Agent (Claude Opus 5)</t>
+        </is>
+      </c>
       <c r="S68" s="47" t="n"/>
+      <c r="T68" s="26" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="U68" s="26" t="inlineStr">
+        <is>
+          <t>DEV-346</t>
+        </is>
+      </c>
+      <c r="V68" s="26" t="inlineStr">
+        <is>
+          <t>1773 → 1791 (+18)</t>
+        </is>
+      </c>
+      <c r="W68" s="26" t="inlineStr">
+        <is>
+          <t>Không đo trên kho cũ được: chưa dự án nào trong du-lieu/ có tiêu chí unit test (loại hiện vật criteria:unit-* vừa mới tồn tại), nên phép đo ở đây là 18 ca chạy trình biên dịch C THẬT trên máy: tệp test in {"do":{"T1":300}} với ngưỡng &lt;=255 → EIDE phán 1 ca HỎNG và câu giải thích mang con số 300. Ca âm: không nêu tiêu chí thì hành vi y như cũ (6 ca test.run trong test_xay_dung.py giữ nguyên, không phải nới ca nào).</t>
+        </is>
+      </c>
+      <c r="X68" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+      <c r="Y68" s="26" t="inlineStr">
+        <is>
+          <t>Phá lại 24/24, lượt đầu 17/24. Bảy chỗ LỌT: năm câu 'nói ra' tôi viết rồi không canh (ma_tieu_chi vào hiện vật, tiêu chí 0 assert, cổng E4023, E4024-ghi-kho-trước, _kiem_assert bị nới), và HAI ca kiểm xanh nhờ một DÒNG KHÁC — kiểm `"TỰ KHAI" in str(kh)` cả khối nên vẫn xanh khi phá chữ ấy ở dòng Kết luận, vì summary cũng chứa nó. · Một phép phá của tôi VÔ HIỆU: `[] or [[…]]` không đổi gì, báo LỌT oan. · Thêm E4023 cho đường unit test (kế hoạch không nêu). · Phải sửa cả surfaces.py, ngoài danh sách tệp chạm tới: test.run ghi vào loại sim_result nên hiện ở khối của sim.run, và dòng Kết luận ở đó nói 'chương trình mô phỏng tự kiểm' cho MỌI lượt. · Chưa lượt Agent nào gọi.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="79.5" customHeight="1" s="27">
       <c r="A69" s="46" t="inlineStr">
@@ -14234,7 +15504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15075,7 +16345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15530,7 +16800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Cất việc: trạng thái 18/106 vào Excel, và chỗ dừng vào toi-uu/DANG-LAM.md
Việc #18 M4-02 đã chốt và gộp main. Không việc nào đang dở.

Excel: sheet mới "Tiến độ 08-10-2026 (toi)" (18 xong · 0 đang làm · 88 chưa), cột
Q, T–Y của dòng M4-02, ô "Cờ tính năng mới" 7 → 8, và hai dòng mới trong khối "Lỗi
tìm thấy trong CHÍNH PHÉP ĐO của tôi".

DANG-LAM.md: chỗ dừng là #19 M4-05, và "bảy thứ phải đọc trước khi gõ" — thêm hai
bài học của M4-02: kiểm lại chính phép phá của mình (ba phép vô hiệu trong hai
nhiệm vụ liền), và một luật policy mới trỏ tới nhóm dữ kiện chưa khai thì DỪNG CẢ
LƯỢT chứ không phải "không nổ". Thêm một việc còn mở: POL-N6-sua-test chưa nổ trên
một phiên thật nào, vì hook của nó cấp dữ kiện cho lời gọi SẮP xảy ra nên không
soát lại được phiên đã lưu.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -11,13 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 07-10-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026 (chiều)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 08-10-2026 (toi)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục tối ưu" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -2099,17 +2100,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -5385,7 +5386,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="59" t="inlineStr">
         <is>
@@ -5584,6 +5584,1313 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" style="27" min="1" max="1"/>
+    <col width="66" customWidth="1" style="27" min="2" max="2"/>
+    <col width="24" customWidth="1" style="27" min="3" max="3"/>
+    <col width="8" customWidth="1" style="27" min="4" max="4"/>
+    <col width="11" customWidth="1" style="27" min="5" max="5"/>
+    <col width="16" customWidth="1" style="27" min="6" max="6"/>
+    <col width="34" customWidth="1" style="27" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>TIẾN ĐỘ ĐỢT TỐI ƯU TÁC TỬ — chốt tối 08/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Mỗi dòng 'Xong' đều có: mục DEV-LOG tra lại được · số ca kiểm trước→sau · một con số đo trên dữ liệu thật · phần còn nợ. Cột chi tiết nằm ở sheet “Danh mục tối ưu”, cột T–Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Tổng quan</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Số việc</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Xong (đã gộp vào main, đã đẩy)</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>18 việc đầu của Giai đoạn 1, theo đúng thứ tự # của kế hoạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Đang làm (chưa commit)</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>không việc nào đang dở</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="n">
+        <v>88</v>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>88 việc còn lại trong 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="n">
+        <v>106</v>
+      </c>
+      <c r="C8" s="61" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>Phép đo của cả đợt</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>Trước (06/10)</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Sau (08/10)</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị Python (pytest -q)</t>
+        </is>
+      </c>
+      <c r="B11" s="63" t="inlineStr">
+        <is>
+          <t>1 610</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>1 816</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>+206 ca so với 06/10; không ca cũ nào đỏ ở bất kỳ bước nào</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị giao diện (swift test)</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>không nhiệm vụ nào đụng ui/ — kiểu khối A2.2 dùng “table”, Swift đã dựng được</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="63" t="inlineStr">
+        <is>
+          <t>kiem_tai_lieu.py</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ LỆCH CHẮC CHẮN cả hai lượt. Hôm nay nó bắt đúng chuyện cần bắt: hai công cụ mới làm README lệch số công cụ 127 → 129, và số 'cần đọc lại' nhảy 11 → 15 → về 11 sau khi sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>thu_sch.py (cờ schematic bật)</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>chạy ở M3-03 và M3-04, không tụt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Mục DEV-LOG mới</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330 → DEV-347</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>18 mục, mỗi việc một mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>Cờ tính năng mới</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>1 (schematic)</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>7 cờ mới, TẤT CẢ mặc định TẮT. Cờ thứ 7 là SIM_RUNNER_GIOI_HAN (M4-02) — nó giới hạn fs.write của sim-runner trong sim/; hàng rào chính của M4-02 (POL-N6-sua-test) thì KHÔNG sau cờ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>Mã lỗi mới</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>E4031 · E4032 · E6012 · E4033 · E4024</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>M4-02 không thêm mã nào: nó DÙNG LẠI E5006 cho cổng ghi của sim-runner. E4033 (M3-18), E4024 (M4-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>Mảng</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>Ưu tiên</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>DEV-LOG</t>
+        </is>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Ca kiểm</t>
+        </is>
+      </c>
+      <c r="G19" s="59" t="inlineStr">
+        <is>
+          <t>Cờ mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>M1-01</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330</t>
+        </is>
+      </c>
+      <c r="F20" s="63" t="inlineStr">
+        <is>
+          <t>105/309 phiên thật có lịch sử tự mâu thuẫn — 255 chỗ (156 kết quả thứ hai cùng id, 74 message chen giữa, 24 kết quả lạc lượt, 1 lời gọi không kết quả)</t>
+        </is>
+      </c>
+      <c r="G20" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>M1-02</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>DEV-331</t>
+        </is>
+      </c>
+      <c r="F21" s="63" t="inlineStr">
+        <is>
+          <t>lược đồ công cụ thật: 25 869 token/lời gọi (trần tool_schema=4000 chưa dòng mã nào đọc). Cờ bật: 4 475 token, giảm 82,7 %; 73 → 18 công cụ</t>
+        </is>
+      </c>
+      <c r="G21" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>M1-03</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
+        <is>
+          <t>DEV-332</t>
+        </is>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>1 822 lời gọi của tác tử con trong 26 phiên thật, 0 lần qua lớp luật. Toàn công cụ đọc trừ một build.compile — lỗ hổng chưa bị bước vào, không phải được canh</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>M2-01</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>DEV-333</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>kịch bản 3 REQ + 3 phương án + 3 tiêu chí + 3 tệp: sửa MỘT REQ làm 9 hiện vật STALE → còn 3. Phép đo đầu ra 6→2 vì bị hàng rào E4020 chặn, đã sửa kịch bản đo</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="inlineStr">
+        <is>
+          <t>TRUY_VET — TẮT (phần nền chạy cả khi tắt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>M2-02</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E24" s="63" t="inlineStr">
+        <is>
+          <t>DEV-334</t>
+        </is>
+      </c>
+      <c r="F24" s="63" t="inlineStr">
+        <is>
+          <t>63 kho thật: 5/37 REQ có ít nhất một phép đo; 27 chưa có phương án nào nhận; 0 REQ đi hết chuỗi. Cột 'Mã nguồn' trống ở MỌI dự án vì hien_thuc_req vừa mới tồn tại</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="inlineStr">
+        <is>
+          <t>REQ_PHU — TẮT (khối A2.2 trên tab không phụ thuộc cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>M2-03</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E25" s="63" t="inlineStr">
+        <is>
+          <t>DEV-335</t>
+        </is>
+      </c>
+      <c r="F25" s="63" t="inlineStr">
+        <is>
+          <t>37 REQ thật: 25 sạch (67 %), 11 thiếu tiêu chí đo được, 2 có từ mơ hồ. Lần đo đầu ra 3 từ mơ hồ, một là kêu oan ('ít nhất 2 lần' là mức đo được) — đã vá</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="inlineStr">
+        <is>
+          <t>REQ_CHAT_LUONG — TẮT (module yeu_cau.py luôn có)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>M2-06</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="inlineStr">
+        <is>
+          <t>DEV-336</t>
+        </is>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>sổ cái thật: 26 lần đánh dấu 'xong' ngay sau một lần ghi mã, 19 lần (73 %) không có phép kiểm nào đạt ở giữa. Phép đo đầu ở mức dự án ra 0 — đúng nhưng đo sai câu hỏi</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="inlineStr">
+        <is>
+          <t>KE_HOACH_CONG_KIEM — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>M2-08</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="inlineStr">
+        <is>
+          <t>DEV-337</t>
+        </is>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>185 tệp .c thật: 1 758 → 1 786 hàm thấy được (+28 hàm trước đây VÔ HÌNH: 8 ngắt + 20 bị regex tham lam nuốt). 78 hàm nay gắn nhãn 'isr', 70 trong đó vốn đã có trong danh sách</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>DEV-338</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mô hình mạch thật — và lý do đáng hơn con số: 3 kho CÓ Fact v_max thì KHÔNG có mô hình mạch, 5 kho có mạch thì không có Fact ấy; thêm nữa Fact dùng chủ thể chip:X mà ERC không tra tiền tố đó</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E29" s="63" t="inlineStr">
+        <is>
+          <t>DEV-339</t>
+        </is>
+      </c>
+      <c r="F29" s="63" t="inlineStr">
+        <is>
+          <t>8 phát hiện trên 5 mạch thật (6 nguon_khong_cap + 2 net_mot_chan), trong đó net clock I2C nối đúng một chân. SÁU trong tám là 'mô hình chưa khai' chứ không phải 'mạch sai'. robot-canbang: 107 Port lá, KHÔNG Port nào là power_out</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E30" s="63" t="inlineStr">
+        <is>
+          <t>DEV-340</t>
+        </is>
+      </c>
+      <c r="F30" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mạch thật — và đây là con số ĐÚNG (hai lỗi này catastrophic, không bo nào sống tới lúc lưu kho). Đã CẤY hai bộ cấp vào bản sao kho robot-canbang để chứng minh luật sống: nổ đúng 1 blocker trên net +5V thật</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>M3-07</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E31" s="63" t="inlineStr">
+        <is>
+          <t>DEV-341</t>
+        </is>
+      </c>
+      <c r="F31" s="63" t="inlineStr">
+        <is>
+          <t>Fact tới được ERC: 5 → 17 (+12). Ba kho có Fact datasheet thì TOÀN BỘ mang chủ thể chip:, tức trước đó không một Fact nào tới được ERC. Độ phủ 5 mạch thật nay đọc được</t>
+        </is>
+      </c>
+      <c r="G31" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>M3-10</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E32" s="63" t="inlineStr">
+        <is>
+          <t>DEV-342</t>
+        </is>
+      </c>
+      <c r="F32" s="63" t="inlineStr">
+        <is>
+          <t>chi phí đo thật: mạch lớn nhất trong kho 187 nút → ERC 7,6 ms mỗi lần ghi. Trần 2000 nút, vượt thì NÓI RA chứ không im lặng bỏ qua</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="inlineStr">
+        <is>
+          <t>ERC_TU_DONG — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>M3-12</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E33" s="63" t="inlineStr">
+        <is>
+          <t>DEV-343</t>
+        </is>
+      </c>
+      <c r="F33" s="63" t="inlineStr">
+        <is>
+          <t>846 bản ghi mô phỏng thật: regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 (testbench dự án in 'KET QUA: PASS' — nhãn đứng TRƯỚC từ khoá). Nới đúng một chỗ → 846/846 khớp, vẫn bắt đủ bốn ca PASS giả</t>
+        </is>
+      </c>
+      <c r="G33" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="64" t="inlineStr">
+        <is>
+          <t>M3-13</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="inlineStr">
+        <is>
+          <t>DEV-344</t>
+        </is>
+      </c>
+      <c r="F34" s="64" t="inlineStr">
+        <is>
+          <t>testbench Verilog THẬT của bài 3: tb_pcpi_dot4 1/1, tb_pcpi_mac 1/1, tb_pcpi_vmini không đo được (tb gọi bản bram HAI CỔNG đã bị bỏ 02/10) — mẫu số là TỆP, không phải phép phá</t>
+        </is>
+      </c>
+      <c r="G34" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>M3-18</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="inlineStr">
+        <is>
+          <t>DEV-345</t>
+        </is>
+      </c>
+      <c r="F35" s="64" t="inlineStr">
+        <is>
+          <t>6 cặp (mạng cổng, .cst) thật → 1 chỗ CHẶN: blinky của riscv-tn20k-b dựng bitstream 4,6 MB với chân đồng hồ do nextpnr tự chọn (rơi đúng chân 4 — bằng may). Cả 7 tệp .cst thật đọc hết, 0 lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="G35" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B36" s="64" t="inlineStr">
+        <is>
+          <t>M4-01</t>
+        </is>
+      </c>
+      <c r="C36" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D36" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E36" s="64" t="inlineStr">
+        <is>
+          <t>DEV-346</t>
+        </is>
+      </c>
+      <c r="F36" s="64" t="inlineStr">
+        <is>
+          <t>18 ca chạy trình biên dịch C thật: tệp test in số đo {"T1":300} với ngưỡng &lt;=255 → EIDE phán 1 ca HỎNG. Chưa kho cũ nào có tiêu chí unit test để đo lại trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="G36" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B37" s="64" t="inlineStr">
+        <is>
+          <t>M4-02</t>
+        </is>
+      </c>
+      <c r="C37" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D37" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E37" s="64" t="inlineStr">
+        <is>
+          <t>DEV-347</t>
+        </is>
+      </c>
+      <c r="F37" s="64" t="inlineStr">
+        <is>
+          <t>25 ca dựng đúng trạng thái thật (tệp test 3 ca, 1 ca đỏ, hiện vật dat=False) → fs.write còn 1 ca thì test.weakened=True. Và hàng rào cũ criteria.has_result chưa bao giờ nổ ngoài sim-01</t>
+        </is>
+      </c>
+      <c r="G37" s="64" t="inlineStr">
+        <is>
+          <t>SIM_RUNNER_GIOI_HAN — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="59" t="inlineStr">
+        <is>
+          <t>Việc còn MỞ (ngoài 88 việc chưa làm)</t>
+        </is>
+      </c>
+      <c r="B39" s="59" t="inlineStr">
+        <is>
+          <t>Vì sao còn mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="63" t="inlineStr">
+        <is>
+          <t>Bảy cờ mới đều còn TẮT</t>
+        </is>
+      </c>
+      <c r="B40" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU · TRUY_VET · REQ_PHU · REQ_CHAT_LUONG · KE_HOACH_CONG_KIEM · ERC_TU_DONG · SIM_RUNNER_GIOI_HAN. Cả bảy đổi thứ Agent nhìn thấy, đọc, hoặc LÀM ĐƯỢC mỗi lượt, nên chỉ bộ 76 ca chạy hai chế độ mới nói được chúng làm Agent khá hơn hay tệ hơn. Bộ ấy tốn tiền mô hình nên §3.0 bắt hỏi người dùng trước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="63" t="inlineStr">
+        <is>
+          <t>kiem_cap_goi_tra() chưa thành hàng rào</t>
+        </is>
+      </c>
+      <c r="B41" s="63" t="inlineStr">
+        <is>
+          <t>Soát được mọi phiên đã lưu, nhưng chưa hook nào gọi nó tự động — bắt được chuyện cũ, chưa chặn được chuyện mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="63" t="inlineStr">
+        <is>
+          <t>Luật ERC quá áp chưa nổ trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="B42" s="63" t="inlineStr">
+        <is>
+          <t>Đường dẫn đã thông ở M3-07, nhưng ba kho có Fact điện áp thì không có mô hình mạch, và ngược lại. Phải chờ một dự án có cả hai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="63" t="inlineStr">
+        <is>
+          <t>Cột “Mã nguồn” của ma trận truy vết trống ở mọi dự án</t>
+        </is>
+      </c>
+      <c r="B43" s="63" t="inlineStr">
+        <is>
+          <t>Nó đọc hien_thuc_req — trường vừa mới tồn tại, chưa tệp nào trên đĩa từng khai. Nên “chưa hiện thực” ở đó nghĩa là “chưa ai KHAI”, không phải “chưa ai viết”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="63" t="inlineStr">
+        <is>
+          <t>Lỗi _go_dau trong src/eide/tools/design.py</t>
+        </is>
+      </c>
+      <c r="B44" s="63" t="inlineStr">
+        <is>
+          <t>Viết .replace('d','d') nên 'ổn định' và 'ON DINH' không khớp nhau. Hàm ấy đang dùng cho một phép kiểm an toàn (người có thật sự chọn không). Tìm thấy ở M2-03, CHƯA sửa vì ngoài phạm vi — cần bộ ca kiểm riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="63" t="inlineStr">
+        <is>
+          <t>subagent req-critic (bước 4 của M2-03)</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="inlineStr">
+        <is>
+          <t>Kế hoạch ghi “tuỳ chọn, gộp M2-13”. Chưa làm, đúng theo kế hoạch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="63" t="inlineStr">
+        <is>
+          <t>Hai luật kiểm chân FPGA chưa có dữ liệu để nổ</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="inlineStr">
+        <is>
+          <t>chan_lech_kit và io_type_lech_bank cần Fact chân kit. Không kho nào trong repo có Fact pin:tangnano20k.* hay khoá vccio — nên hôm nay chỉ 3 trong 5 luật của M3-18 kết luận được gì trên dữ liệu thật. Cùng hình dạng với luật ERC quá áp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="63" t="inlineStr">
+        <is>
+          <t>Một bitstream cũ đã dựng với chân đồng hồ tự chọn</t>
+        </is>
+      </c>
+      <c r="B47" s="63" t="inlineStr">
+        <is>
+          <t>blinky của du-lieu/riscv-tn20k-b — xem DEV-345 và README §8. Không sửa hiện vật cũ: đó là dữ liệu của những lượt đo đã chốt. Từ nay phép kiểm chặn trước nextpnr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="63" t="inlineStr">
+        <is>
+          <t>Ba công cụ mới nhất chưa lượt Agent nào GỌI</t>
+        </is>
+      </c>
+      <c r="B48" s="63" t="inlineStr">
+        <is>
+          <t>hdl.sensitivity · hdl.constraints_check · test.criteria. Mã của cả ba đã chạy trên hiện vật thật, nhưng đó là tôi gọi hàm, không phải tác tử gọi công cụ. README §8 đếm cả ba vào phần chưa dùng thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="63" t="inlineStr">
+        <is>
+          <t>POL-N6-sua-test chưa nổ trên một phiên thật nào</t>
+        </is>
+      </c>
+      <c r="B49" s="63" t="inlineStr">
+        <is>
+          <t>Hook sua_test_sau_do cấp dữ kiện cho lời gọi SẮP xảy ra, nên không soát lại được phiên đã lưu — khác mọi phép đo trước của đợt này. Nó đã có 25 ca kiểm và phá lại 27/27, nhưng chưa lượt tác tử thật nào chạm vào nó. Cùng hình dạng với ba luật kiểm thiếu dữ liệu ở trên, chỉ khác lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="59" t="inlineStr">
+        <is>
+          <t>Lỗi tìm thấy trong CHÍNH PHÉP ĐO của tôi</t>
+        </is>
+      </c>
+      <c r="B51" s="59" t="inlineStr">
+        <is>
+          <t>Lộ ra ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="63" t="inlineStr">
+        <is>
+          <t>Kịch bản đo bị hàng rào của sản phẩm chặn (ghi tệp chưa đọc, E4020) và trả về một con số hợp lý thay vì nổ — 6→2 trông đẹp y như 9→3 đúng</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="inlineStr">
+        <is>
+          <t>M2-01 · DEV-333</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm dựng trên điều tôi tự nhớ sai: “thiết” bỏ dấu KHÔNG chứa “it”; chỗ va thật là bit/unit/init/exit</t>
+        </is>
+      </c>
+      <c r="B53" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá dài ĐÚNG BẰNG mã gốc (0.6 → 0.0) nên __pycache__ cũ còn hiệu lực — phép đo chạy mã khác với mã trong tệp</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="63" t="inlineStr">
+        <is>
+          <t>Phép đo trả lời ĐÚNG một câu hỏi KHÁC: đếm ở mức dự án ra 0 chỗ cần chặn; câu phải hỏi là “lần ghi NÀY đã được kiểm chưa” → 19/26</t>
+        </is>
+      </c>
+      <c r="B55" s="63" t="inlineStr">
+        <is>
+          <t>M2-06 · DEV-336</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm RỖNG: dàn dựng không có net đất nào, nên nó xanh cả khi tôi bỏ hẳn phép bỏ qua net đất</t>
+        </is>
+      </c>
+      <c r="B56" s="63" t="inlineStr">
+        <is>
+          <t>M3-01 · DEV-338</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="63" t="inlineStr">
+        <is>
+          <t>Hai phép phá chỉ ra THIẾT KẾ sai, không chỉ ca kiểm yếu (miễn net đất quá rộng; nhánh iout_max chưa ca nào chạm tới)</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="inlineStr">
+        <is>
+          <t>M3-03 · DEV-339</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá của tôi cũng SAI, và ca âm xanh vì lý do khác — hai cái sai che nhau</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="inlineStr">
+        <is>
+          <t>M3-07 · DEV-341</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm đo chính câu lệnh của mình (đặt bộ đếm = 3 rồi khẳng định nó khác rỗng, trong khi thực tế nó rỗng)</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="inlineStr">
+        <is>
+          <t>M3-10 · DEV-342</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="63" t="inlineStr">
+        <is>
+          <t>Regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 bản ghi thật; và ba ca kiểm xanh vì lý do sai (tệp giả dùng $4 thay $3; “FAILED” chứa “FAIL”)</t>
+        </is>
+      </c>
+      <c r="B60" s="63" t="inlineStr">
+        <is>
+          <t>M3-12 · DEV-343</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="63" t="inlineStr">
+        <is>
+          <t>"Phá lại thì đỏ 6/6" sai về TẬP, không sai về số: sáu phép phá ấy chọn đúng sáu chỗ đã có ca canh. Phá bằng tập rộng hơn ra 7/9.</t>
+        </is>
+      </c>
+      <c r="B61" s="63" t="inlineStr">
+        <is>
+          <t>M3-13 · DEV-344</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="63" t="inlineStr">
+        <is>
+          <t>409 'blocker' gần như toàn bộ từ một cặp vô nghĩa (mạng cổng của lõi CPU tổng hợp riêng, không bao giờ đem đặt-đi dây). Con số thật là 1.</t>
+        </is>
+      </c>
+      <c r="B62" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="63" t="inlineStr">
+        <is>
+          <t>Phép quét tệp .cst thật chỉ thu 4 trong 7 tệp mà ca kiểm vẫn xanh — câu 'mọi tệp .cst thật đều đọc được' nói về phần phép quét chạm tới.</t>
+        </is>
+      </c>
+      <c r="B63" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="63" t="inlineStr">
+        <is>
+          <t>Một ca kiểm và một phép phá nhắm hai NHÁNH khác nhau, nên ca mới xanh mà phép phá vẫn LỌT. Mất một lượt mới thấy.</t>
+        </is>
+      </c>
+      <c r="B64" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm xanh nhờ một DÒNG KHÁC: kiểm `"TỰ KHAI" in str(kh)` cả khối nên vẫn xanh khi phá chữ ấy ở dòng Kết luận — summary cũng chứa nó. Phép phá bắt được, ca kiểm thì không.</t>
+        </is>
+      </c>
+      <c r="B65" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="63" t="inlineStr">
+        <is>
+          <t>Một phép phá VÔ HIỆU: `them = [] or [[…]]` không đổi hành vi, nên nó báo LỌT oan và suýt làm tôi viết ca kiểm cho một chỗ vốn đã được canh.</t>
+        </is>
+      </c>
+      <c r="B66" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="63" t="inlineStr">
+        <is>
+          <t>HAI phép phá liền nhau VÔ HIỆU ở cùng một dòng: `cu = cu or ""` không đổi hành vi, rồi bỏ is_file() cũng không vì except OSError bắt FileNotFoundError. Phải bỏ cả hai lớp phòng mới phá được.</t>
+        </is>
+      </c>
+      <c r="B67" s="63" t="inlineStr">
+        <is>
+          <t>M4-02 · DEV-347</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="63" t="inlineStr">
+        <is>
+          <t>Một luật mới trỏ tới nhóm dữ kiện chưa khai thì DỪNG CẢ LƯỢT bằng ValueError, không phải 'không nổ' — và nhóm `criteria` của hàng rào N6 cũ cũng chưa bao giờ được khai.</t>
+        </is>
+      </c>
+      <c r="B68" s="63" t="inlineStr">
+        <is>
+          <t>M4-02 · DEV-347</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11933,11 +13240,45 @@
       </c>
       <c r="Q69" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R69" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R69" s="47" t="inlineStr">
+        <is>
+          <t>Agent (Claude Opus 5)</t>
+        </is>
+      </c>
       <c r="S69" s="47" t="n"/>
+      <c r="T69" s="26" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="U69" s="26" t="inlineStr">
+        <is>
+          <t>DEV-347</t>
+        </is>
+      </c>
+      <c r="V69" s="26" t="inlineStr">
+        <is>
+          <t>1791 → 1816 (+25)</t>
+        </is>
+      </c>
+      <c r="W69" s="26" t="inlineStr">
+        <is>
+          <t>Không có dữ liệu cũ để đo lại trên: hook này cấp dữ kiện cho lời gọi SẮP xảy ra, không soát lại phiên đã lưu. Phép đo là 25 ca dựng đúng trạng thái thật: tệp test 3 ca với 1 ca đỏ trên đĩa + hiện vật sim_result dat=False trong kho → fs.write còn 1 ca thì test.weakened=True và test.doi_gi nói '7 chỗ canh → 3'. Và một phép đo trên chính hàng rào cũ: criteria.has_result tra cứng sim_result:can-bang, nên POL-N6-doi-tieu-chi CHƯA BAO GIỜ nổ cho sim-ntc hay unit-* — luật viết đúng, đường dẫn tới nó đứt.</t>
+        </is>
+      </c>
+      <c r="X69" s="26" t="inlineStr">
+        <is>
+          <t>SIM_RUNNER_GIOI_HAN — TẮT (hàng rào chính POL-N6-sua-test thì KHÔNG sau cờ)</t>
+        </is>
+      </c>
+      <c r="Y69" s="26" t="inlineStr">
+        <is>
+          <t>Phá lại 27/27, lượt đầu 22/27. · PHÁT HIỆN ngoài phạm vi kế hoạch: một luật trỏ tới nhóm dữ kiện chưa khai thì DỪNG CẢ LƯỢT bằng ValueError, không phải 'không nổ' — _env có danh sách 'nhóm phải luôn tồn tại' và nhóm `test` không có trong đó, nên luật mới làm mọi fs.write đổ. Mở ra thì thấy `criteria` cũng chưa bao giờ có trong danh sách ấy. · HAI phép phá của tôi vô hiệu ở cùng một dòng: `cu = cu or ""` không đổi hành vi, rồi bỏ is_file() cũng không vì except OSError bắt FileNotFoundError. Lần thứ hai liền sau M4-01. · Bốn chỗ LỌT còn lại: tiền tố unit-, số chỗ canh không đổi, testbench ngoài thư mục test/, và luật (khác hook) cho test.criteria.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="90.75" customHeight="1" s="27">
       <c r="A70" s="46" t="inlineStr">
@@ -15504,7 +16845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16345,7 +17686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16800,7 +18141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Điền bằng chứng việc #24 (M4-09) vào Danh mục tối ưu
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2105,17 +2105,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3868,7 +3868,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="27">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -10946,11 +10945,45 @@
       <c r="P76" s="47" t="n"/>
       <c r="Q76" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R76" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R76" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S76" s="47" t="n"/>
+      <c r="T76" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U76" s="26" t="inlineStr">
+        <is>
+          <t>DEV-353</t>
+        </is>
+      </c>
+      <c r="V76" s="26" t="inlineStr">
+        <is>
+          <t>1 896 → 1 901 (5 ca mới trong tests/test_tu_phat_hien_sai.py: TC-M4-09-01, TC-M4-09-02 cả hai mặt firmware/verifier, TC-M4-09-03, và ca mặc định của getattr). Ca CŨ test_da_goi_verifier_roi_thi_thoi đã sửa vì nó khoá đúng hành vi SAI (§3.2). Phá lại thì đỏ: 10/12 — hai chỗ LỌT đã kiểm lại là KHÔNG đổi hành vi (bỏ res.ok là guard chết vì _one_tool return sớm; so lỏng 'verifier' in ten vô hiệu vì trong tám tên SUBAGENT chỉ verifier chứa chuỗi ấy)</t>
+        </is>
+      </c>
+      <c r="W76" s="26" t="inlineStr">
+        <is>
+          <t>68 sổ cái dự án (26 sổ có task.run, 257 lời gọi: verifier 253 · code-analyst 2 · firmware 1 · sim-runner 1). Hook Stop ghi lại chính checks của nó, nên đếm được: 41 lượt hook khai tu_kiem_da_chay (đã IM), và 1 trong 41 lượt ấy KHÔNG có task.run(verifier) nào — robot-sinhvien2 run-007, nơi lời gọi task.run(code-analyst) nằm TRƯỚC fs.edit vào ISR(TIMER2_COMPA_vect), build.compile và fs.write sim/dump_isr.c. Quét theo hình dạng ra 2 lượt: thêm rtos-sinhvien run-026, lượt có cả target.flash.</t>
+        </is>
+      </c>
+      <c r="X76" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+      <c r="Y76" s="26" t="inlineStr">
+        <is>
+          <t>Không còn nợ tiêu chí nào. Ghi chú thiết kế: câu 'còn việc chưa ai kiểm chưa' vẫn đọc SỔ CÁI (xuyên phiên, co_viec_chua_kiem không đổi); chỉ câu 'verifier có chạy trong LƯỢT này không' mới dùng cờ trên ctx — ctx sinh ra và chết cùng lượt nên nó là vật đúng để hỏi.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="57" customHeight="1" s="27">
       <c r="A77" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M4-11] STALE theo tệp + chặn tuyên xong khi còn STALE + hồi quy nhẹ sau cờ
trước 1 901 ca / sau 1 929 ca

`test.run`/`sim.run` gọi `store.apply` KHÔNG có `deps=`, nên chuỗi mặc định §E5.4 đánh
STALE mọi kết quả test/sim khi sửa bất kỳ tệp mã nào. Lớp đọc (`ha_nguon_cua`) đã đúng
từ M2-01 — ba ca kiểm đầu của bảng TC xanh sẵn; chỗ đứt là lớp GHI.

`upstream` là bao đóng `#include "..."` cục bộ, không phải danh sách tệp đưa cho trình
biên dịch: `robot-sinhvien2` lưu `tep_nguon = ['sim/test_balance.c']` mà tệp ấy
`#include "../firmware/pid.c"`, `motor.c`, `filter.c`.

Đo trên 9 kho thật: bán kính STALE 107 → 49 lần (58/107 là cáo buộc oan).
Hook `ket_qua_stale` (không cờ) chặn lời tuyên xong khi còn kết quả lỗi thời.
Hồi quy nhẹ sau cờ `HOI_QUY_NEN` (TẮT) — mách con số, KHÔNG xoá nhãn STALE.

Phá lại thì đỏ 24/32 → 31/34; ba chỗ LỌT còn lại không đổi hành vi. DEV-354.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2105,17 +2105,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -11155,11 +11155,45 @@
       </c>
       <c r="Q78" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R78" s="47" t="n"/>
+          <t>Xong (một tiêu chí CHƯA đạt)</t>
+        </is>
+      </c>
+      <c r="R78" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S78" s="47" t="n"/>
+      <c r="T78" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U78" s="26" t="inlineStr">
+        <is>
+          <t>DEV-354</t>
+        </is>
+      </c>
+      <c r="V78" s="26" t="inlineStr">
+        <is>
+          <t>1 901 → 1 929 (28 ca mới trong tests/test_hoi_quy.py). Phá lại thì đỏ: 24/32 lượt đầu → 31/34 sau khi thêm bảy ca kiểm và hai phép phá GỘP. Ba chỗ LỌT còn lại đã kiểm lại là KHÔNG đổi hành vi: bỏ ung.is_file() (p.is_file() vẫn lọc), trần quay lại đếm len(xong) (dedupe vẫn làm hàng đợi cạn), bỏ res.ok (guard chết vì _one_tool return sớm). Hai lớp phòng độc lập thì CHỈ phép phá gộp nói được có ca canh hay không — gộp dedupe + trần-đếm-lượt thì vòng lặp không dừng, và ca luồng-có-đồng-hồ biến nó thành chữ ĐỎ trong 8 giây thay vì một lượt treo 120 giây.</t>
+        </is>
+      </c>
+      <c r="W78" s="26" t="inlineStr">
+        <is>
+          <t>9 kho THẬT: bán kính STALE của kết quả test/sim khi sửa một tệp mã 107 lần → 49 lần, tức 58/107 (54 %) là cáo buộc OAN. Chi tiết: robot-canbang 6→3 · robot-sinhvien 14→10 · robot-sinhvien2 14→5 · robot-tu-can-bang 24→13 · rtos-sinhvien 30→8 · stm32f469-freertos 12→6 · usecase/uc03 3→1 · usecase/uc11 4→3. Và chính dữ liệu thật bác bước 1 của kế hoạch: robot-sinhvien2 lưu tep_nguon = ['sim/test_balance.c'] MỘT tệp, mà tệp ấy #include '../firmware/pid.c', motor.c, filter.c — nên upstream phải là bao đóng #include, không phải danh sách tệp đưa cho trình biên dịch. Bao đóng ra đúng 5 mắt.</t>
+        </is>
+      </c>
+      <c r="X78" s="26" t="inlineStr">
+        <is>
+          <t>HOI_QUY_NEN — mặc định TẮT (phần deps.upstream + hook ket_qua_stale KHÔNG sau cờ)</t>
+        </is>
+      </c>
+      <c r="Y78" s="26" t="inlineStr">
+        <is>
+          <t>Tiêu chí 'số lần tuyên xong với kết quả STALE = 0' CHƯA ĐẠT: sổ cái ghi lời gọi công cụ và checks của hook, nhưng KHÔNG ghi trạng thái kho tại thời điểm ấy — nên khác mọi phép đo khác của đợt, nó không soát lại được phiên đã lưu. Đóng nó cần PHÁT LẠI phiên mẫu với hook mới, tức lời gọi mô hình thật (§3.0 bắt hỏi anh Công trước). Và kế hoạch SAI chỗ: nó bảo sửa deps.ha_nguon_cua, nhưng ba ca kiểm đầu XANH SẴN — lớp đọc đã đúng từ M2-01; chỗ đứt là lớp GHI (test.run/sim.run gọi store.apply không có deps). Lỗi tìm thấy trong chính mã vừa viết: trần của _khep_include đếm len(xong) nên không chặn được vòng #include vô hạn — phép phá treo 900 giây thay vì đỏ; nay trần đếm LƯỢT.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="68.25" customHeight="1" s="27">
       <c r="A79" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M5-03] Bộ đọc SVD → Fact reg:/field: có trích dẫn, và công cụ reg.lookup
trước 1 942 ca / sau 1 950 ca

`phan_loai` khai tệp SVD là ĐẦY ĐỦ, `doc.load` trả `E1001 "chưa có bộ đọc"` — hai câu
trả lời trái nhau cho cùng một tệp, và `grep -rni svd src/` ra đúng hai chỗ: phép phân
loại, và một comment nói "bốn loại đó có công cụ riêng".

`knowledge/svd.py` đọc bằng `xml.etree` (không thêm phụ thuộc): `derivedFrom` cả hai
chiều, `cluster` một cấp kèm offset và tiền tố tên, và cả ba lối khai vị trí bit. Địa
chỉ do MÃ cộng, hex tám chữ số, mỗi Fact kèm trích dẫn `<P>.<R>[.<F>]`.

Hai chỗ chọn phía thận trọng: `baseAddress` hỏng thì bỏ cả ngoại vi, thanh ghi thiếu
`addressOffset` thì bỏ — một địa chỉ bằng `base` là một địa chỉ SAI mà hợp lệ.
Trần `TRAN_DON_VI` nay NÓI RA chỗ nó cắt.

Phá lại thì đỏ 28/34 → 34/34; sáu chỗ LỌT đều là lỗ thật. DEV-355.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2108,13 +2108,13 @@
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
@@ -3868,6 +3868,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="27">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -12431,11 +12432,45 @@
       <c r="P92" s="47" t="n"/>
       <c r="Q92" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R92" s="47" t="n"/>
+          <t>Xong (một tiêu chí CHƯA đạt)</t>
+        </is>
+      </c>
+      <c r="R92" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S92" s="47" t="n"/>
+      <c r="T92" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U92" s="26" t="inlineStr">
+        <is>
+          <t>DEV-355</t>
+        </is>
+      </c>
+      <c r="V92" s="26" t="inlineStr">
+        <is>
+          <t>1 942 → 1 950 (21 ca mới + 1 ca nha_that) trong tests/test_svd.py. Phá lại thì đỏ: 28/34 lượt đầu → 34/34. Sáu chỗ LỌT đều là lỗ THẬT, không chỗ nào vô hiệu: _so trả 0 thay vì None; bỏ lối khai bit thứ ba lsb/msb; thanh ghi thiếu addressOffset vẫn nạp; dem() trả (r,r) vẫn xanh vì ca kiểm chính ra 4 thanh ghi và 4 trường — HAI VẾ TÌNH CỜ BẰNG NHAU; reg.lookup không gom theo chủ thể vẫn xanh vì 25 thanh ghi của ca trần chỉ có MỘT Fact mỗi cái; trần 20 nâng được lên 500 qua tham số. Hai chỗ giữa cùng một hình dạng: phép đo xanh vì DÀN DỰNG làm hai vế trùng nhau, không vì mã đúng.</t>
+        </is>
+      </c>
+      <c r="W92" s="26" t="inlineStr">
+        <is>
+          <t>grep -rni svd src/ TRƯỚC khi sửa ra đúng HAI chỗ: phép phân loại, và một câu comment nói 'bốn loại đó có công cụ riêng' — không có bộ đọc nào. Tức phan_loai khai ĐẦY ĐỦ còn doc.load trả E1001 'chưa có bộ đọc': hai câu trả lời trái nhau cho cùng một tệp. CHƯA đo được trên SVD thật: quét cả máy 09/10/2026 không có tệp .svd nào ngoài tệp do chính bộ kiểm sinh trong tmp.</t>
+        </is>
+      </c>
+      <c r="X92" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần + công cụ mới core=False</t>
+        </is>
+      </c>
+      <c r="Y92" s="26" t="inlineStr">
+        <is>
+          <t>Tiêu chí 'nạp được SVD thật STM32F469, ghi số thanh ghi' CHƯA ĐẠT: máy không có tệp .svd thật nào. Ca test_nap_duoc_SVD_THAT đã viết, đánh nha_that + skipif, dò ~/STM32Cube · ~/.platformio · STM32CubeIDE.app · tai-lieu-tham-khao/ và SKIP. Không tự viết một SVD lớn rồi gọi nó là 'thật' — một bộ đọc chạy đúng trên tệp tự viết chưa nói gì về một tệp có derivedFrom khắp nơi và cluster lồng nhau. reg.lookup là công cụ thứ 132 và CHƯA lượt Agent nào gọi (README §8 đếm nó vào phần chưa dùng thật). Lỗi tìm thấy trong chính mã vừa viết: trần TRAN_DON_VI cắt IM LẶNG — nay doc.load trả da_cat_o_tran và nói ra, vì 'chip không có' và 'chưa nạp tới' dẫn tới hai việc ngược nhau.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="79.5" customHeight="1" s="27">
       <c r="A93" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M5-05] Kiểm thứ nguyên đơn vị + thống nhất khoá khoảng + kiểm cả đường bảng
trước 1 976 ca / sau 1 980 ca

`hop_ly("vdd.max", 25, "°C")` trả `True`: nó quy về đơn vị cơ bản rồi chỉ so ĐỘ LỚN, và
25 lọt khoảng điện áp 0,5–60 V. Một Fact như thế ở tầng BẠC là vế giới hạn của luật ERC
quá áp. Thêm `THU_NGUYEN_KHOA` tra theo tiền tố DÀI NHẤT (ba khoá `i2c.*` có ba thứ
nguyên khác nhau), thêm khoảng cho `fmax`/`ta.*` (hai khoá bộ trích THẬT SỰ sinh ra), và
cho đường hàng bảng đi qua `hop_ly`.

Hai lỗ nữa tìm ra bằng tập phá, ngoài phạm vi kế hoạch: `hop_ly` nổ `TypeError` với giá
trị chuỗi, và đường bảng sinh khoá `flash.max`/`fmax.max` — khoá không chỗ nào đọc, nên
một dung lượng Flash đọc từ BẢNG chưa bao giờ thành hạn mức.

TC-M5-05-04 của kế hoạch xanh sẵn vì `"VDD"` trơn không khớp mẫu nào.

Phá lại thì đỏ 17/21 → 23/24. DEV-356.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2105,17 +2105,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -12642,11 +12642,45 @@
       </c>
       <c r="Q94" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R94" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R94" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S94" s="47" t="n"/>
+      <c r="T94" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U94" s="26" t="inlineStr">
+        <is>
+          <t>DEV-356</t>
+        </is>
+      </c>
+      <c r="V94" s="26" t="inlineStr">
+        <is>
+          <t>1 976 → 1 980 (30 ca mới trong tests/test_don_vi_fact.py). Phá lại thì đỏ: 17/21 lượt đầu → 23/24. Hai chỗ LỌT là LỖ THẬT, thành hai phần sửa thêm: hop_ly NỔ TypeError với giá trị chuỗi (i2c.addr sống sót chỉ vì nó không có khoảng), và hàng bảng tra bằng khoa_goc nên mất phép kiểm KHOẢNG. Hai chỗ còn lại vô hiệu: 'tra tiền tố ngắn nhất trước' không đổi gì vì bảng không có khoá 'i2c' — tức ca kiểm i2c của tôi KHÔNG đo được tính chất nó nói nó đo; và break thay continue thoát một vòng lặp MỘT phần tử.</t>
+        </is>
+      </c>
+      <c r="W94" s="26" t="inlineStr">
+        <is>
+          <t>hop_ly('vdd.max', 25, '°C') trả True trên mã cũ — 25 lọt khoảng điện áp 0,5–60 V. Và TC-M5-05-04 của kế hoạch XANH SẴN vì một lý do khác: 'VDD' trơn không khớp mẫu nào trong _MAU_THONG_SO, nên hàng rỗng vì tên chứ không vì phép kiểm đơn vị. Lỗ thứ hai đo được bằng tập phá: đường BẢNG và đường DÒNG CHỮ sinh HAI khoá khác nhau cho cùng một thông số — flash.size/flash.max, fmax/fmax.max, i2c.addr/i2c.max — và xay_dung._han_muc KHÔNG đọc flash.max, nên một dung lượng Flash đọc từ BẢNG chưa bao giờ thành hạn mức.</t>
+        </is>
+      </c>
+      <c r="X94" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+      <c r="Y94" s="26" t="inlineStr">
+        <is>
+          <t>Không còn nợ tiêu chí nào. Ba khoá bị đổi (flash.max, fmax.max, i2c.max) là ba khoá KHÔNG chỗ nào đọc, nên đổi chúng không làm lệch Fact cũ nào đang khớp với ai — đúng tinh thần dòng 'Không đổi tên khoá mà bộ trích sinh ra' của kế hoạch.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="68.25" customHeight="1" s="27">
       <c r="A95" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M5-07] fact.from_doc: ranh giới token, câu trích nguyên văn, đơn vị đứng sau số
trước 1 993 ca / sau 2 000 ca

Phép kiểm cũ xoá dấu chấm rồi dùng `in`, nên `2.7 V` thành `27v` và `gia_tri="27"` đi
qua — một điện áp 2,7 V vào kho thành 27, mang trích dẫn, mang tầng BẠC. Và phép CHỨA
không ranh giới nên `3` khớp `Table 3`, `180` khớp `1800`, `39` khớp `0.39`.

Bốn phép kiểm mới: `trich` phải có thật trong đoạn · ranh giới token · giá trị ≤2 ký tự
phải kèm `trich` · `don_vi_do` phải đứng ngay sau số và khớp cả token. `source.quote`
nay là chỗ CÓ con số, không phải 200 ký tự đầu đoạn.

Giữ E2006 cho "giá trị không có trong đoạn"; E2008 cho ba lý do MỚI.
Một ca cũ sửa theo §3.2 (nêu `trich` cho giá trị "39").

Phá lại thì đỏ 15/22 → 22/22; cả bảy chỗ LỌT là ca kiểm chưa chạm tới. DEV-357.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2105,17 +2105,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -12848,11 +12848,45 @@
       <c r="P96" s="47" t="n"/>
       <c r="Q96" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R96" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R96" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S96" s="47" t="n"/>
+      <c r="T96" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U96" s="26" t="inlineStr">
+        <is>
+          <t>DEV-357</t>
+        </is>
+      </c>
+      <c r="V96" s="26" t="inlineStr">
+        <is>
+          <t>1 993 → 2 000 (20 ca mới trong tests/test_fact_from_doc.py). Phá lại thì đỏ: 15/22 lượt đầu → 22/22. CẢ BẢY chỗ LỌT là ca kiểm của tôi CHƯA CHẠM TỚI, không chỗ nào vô hiệu — và năm trong bảy chỉ lộ ra khi dàn dựng có đúng hình dạng cần đo: bốn dòng văn bản thêm vào bộ dàn dựng (0.39 phần trăm · 0x27 một mình · '39,' · 100 mA) là thứ biến bảy chữ LỌT thành bảy chữ ĐỎ. Một ca CŨ phải sửa theo §3.2 (nêu `trich` cho giá trị '39').</t>
+        </is>
+      </c>
+      <c r="W96" s="26" t="inlineStr">
+        <is>
+          <t>Phép kiểm cũ: re.sub(r'[\s.,]', '', x) rồi `in`. Nó nhận bừa ở hai chỗ, đo được bằng ca kiểm trên tài liệu thật nạp qua doc.load: '2.7 V' thành '27v' nên gia_tri='27' đi qua; và phép CHỨA không ranh giới nên '3' khớp 'Table 3', '180' khớp '1800', '39' khớp '0.39'. source.quote lưu 200 ký tự ĐẦU đoạn, không phải chỗ có con số — người mở Fact ra xem thấy một đoạn không chứa con số.</t>
+        </is>
+      </c>
+      <c r="X96" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+      <c r="Y96" s="26" t="inlineStr">
+        <is>
+          <t>Không còn nợ tiêu chí nào. HAI chỗ không theo chữ kế hoạch: (1) giữ E2006 cho 'giá trị không có trong đoạn' và dùng E2008 chỉ cho ba lý do MỚI — gộp cả bốn vào một mã là bắt tác tử học một mã cho bốn việc khác nhau, và một ca kiểm cũ đang khoá đúng nghĩa cũ; (2) TC-M5-07-01 viết đúng chữ thì XANH VÌ LÝ DO KHÁC — '27' dài hai ký tự nên luật số-ngắn chặn trước và phép so dấu chấm không bao giờ chạy tới. `trich` KHÔNG thành tham số bắt buộc: giá trị từ 3 ký tự trở lên vẫn gọi được như cũ.</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="79.5" customHeight="1" s="27">
       <c r="A97" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M5-13] Chính sách phong bì cho doc.read/fact.query/fact.extract + _cat_chung cắt phần tử
trước 2 012 ca / sau 2 015 ca

Ba công cụ đọc tri thức không có chính sách riêng, và trần chung bị LÁCH: `_cat_chung`
cắt số phần tử của list (`d[:30]`) mà không cắt từng phần tử, rồi cắt mỗi chuỗi theo
trần của CẢ kết quả. `{"ds": ["y"*20000]*5}` ra 20 000 token qua một cái trần 4 000.

`doc.read`: ≤8 đoạn, 600 ký tự QUANH chỗ khớp `tim` (không lấy đầu đoạn).
`fact.query`/`fact.extract`: ≤30 Fact, bỏ `explain`, giữ `source` gọn.
`_cat_chung`: ngân sách đi xuống theo nhánh, và chỗ gọi chừa 1/4 trần cho vỏ JSON.

Đo trên 23 kho THẬT: một `fact.query` đưa 67 635 → 32 560 token vào ngữ cảnh (−51 %);
`robot-sinhvien` một mình 12 076 → 4 579.

Phá lại thì đỏ 20/23 → 23/23; cả ba chỗ LỌT là dàn dựng làm phép phá vô hiệu. DEV-358.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2108,13 +2108,13 @@
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
@@ -13390,11 +13390,45 @@
       </c>
       <c r="Q102" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R102" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R102" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S102" s="47" t="n"/>
+      <c r="T102" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U102" s="26" t="inlineStr">
+        <is>
+          <t>DEV-358</t>
+        </is>
+      </c>
+      <c r="V102" s="26" t="inlineStr">
+        <is>
+          <t>2 012 → 2 015 (tổng 15 ca mới trong tests/test_mem_a.py). Phá lại thì đỏ: 20/23 lượt đầu → 23/23. Cả BA chỗ LỌT là DÀN DỰNG làm phép phá vô hiệu, không phải mã đúng: không ca nào có hàng bảng nhiều ô; ca âm dựng `source` ĐÃ ĐÚNG hình dạng _gon trả về nên hạ trần kích hoạt cũng không đổi gì; và ca {'ds': [...]} có MỘT khoá nên chia ngân sách cho một là phép đồng nhất. Lần thứ ba liền (M5-03 · M5-07 · M5-13) chỗ LỌT nằm ở bộ dàn dựng.</t>
+        </is>
+      </c>
+      <c r="W102" s="26" t="inlineStr">
+        <is>
+          <t>23 kho THẬT: một lời gọi fact.query không tham số đưa 67 635 token vào ngữ cảnh trước → 32 560 sau (giảm 35 075, tức 51 %). Đo bằng cách bọc hai lần — một lần với chính sách mới, một lần với bảng CHINH_SACH đã bỏ fact.query ra. robot-sinhvien một mình: 30 Fact → 12 076 token cho MỘT lời gọi, nay 4 579 (bốn lời gọi như thế là hết một cửa sổ 48k). Bốn kho nhỏ (1–2 Fact) ra con số y nguyên, đúng như ca âm đòi.</t>
+        </is>
+      </c>
+      <c r="X102" s="26" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+      <c r="Y102" s="26" t="inlineStr">
+        <is>
+          <t>Không còn nợ tiêu chí nào. Lỗi tìm thấy trong chính mã vừa viết: _cat_chung tiêu ĐÚNG ngân sách nó được giao, nên giao cả trần thì shown_tokens nhảy lên 4 024 vì vỏ JSON — một cái trần bị vượt bởi chính phép cắt dựng ra để giữ nó; nay chỗ gọi chừa một phần tư. Bài học gom lại: khi dựng ca kiểm cho một phép CHIA hay một phép CẮT, dàn dựng phải có ít nhất HAI phần tử và chúng phải KHÁC NHAU.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="102" customHeight="1" s="27">
       <c r="A103" s="46" t="inlineStr">

</xml_diff>

<commit_message>
[M5-17] Resume nạp lại bản tóm tắt C2 từ sổ cái + tường thuật cơ học sau cờ
trước 2 015 ca / sau 2 030 ca

`BoNen.tom_tat_hien_tai` chỉ được gán khi nén thành công TRONG tiến trình ấy, nên bản
tóm tắt sống đúng một tiến trình rồi mất — mà nó là NGUỒN DUY NHẤT về đoạn hội thoại đã
bị nén khỏi ngữ cảnh, và nó đã được ghi vào sổ cái từ đầu.

`tom_tat_cuoi_tu_so_cai` duyệt ngược, dừng ở `compact` gần nhất: `ok` → trả bản ấy,
`huy` → trả None (§6.2.3 — huỷ nghĩa là đoạn ấy quay về nguyên văn).
`BanTomTat.tu_dict` đảo `to_dict`, chịu được dữ liệu thiếu khoá.

Phần B sau cờ `RESUME_TUONG_THUAT` (TẮT): tường thuật cơ học phiên trước, 0 token mô
hình — 303/313 phiên thật (96 %) chưa từng chạm ngưỡng nén.

Phá lại thì đỏ 20/23 → 23/23; cả ba chỗ LỌT là ca kiểm chưa chạm tới dòng nó canh.
DEV-359.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -2105,17 +2105,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B53:G53"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -13764,11 +13764,45 @@
       <c r="P106" s="47" t="n"/>
       <c r="Q106" s="48" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="R106" s="47" t="n"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="R106" s="47" t="inlineStr">
+        <is>
+          <t>Claude (Opus 5)</t>
+        </is>
+      </c>
       <c r="S106" s="47" t="n"/>
+      <c r="T106" s="26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="U106" s="26" t="inlineStr">
+        <is>
+          <t>DEV-359</t>
+        </is>
+      </c>
+      <c r="V106" s="26" t="inlineStr">
+        <is>
+          <t>2 015 → 2 030 (18 ca mới trong tests/test_mem_c.py). Phá lại thì đỏ: 20/23 lượt đầu → 23/23. Cả BA chỗ LỌT là ca kiểm CHƯA chạm tới dòng mã nó nói nó canh: chuỗi '`target.flash` → E4040' cũng có ở dòng 'Lỗi cuối cùng' nên assertion xanh qua dòng khác; transcript dàn dựng ngắn hơn trần 1 500 nên bỏ trần không đổi gì; và ca 'transcript hỏng' chạy trên dự án CHỈ CÓ MỘT PHIÊN nên hàm trả rỗng ngay ở bước 'không có phiên trước'. Bốn nhiệm vụ liền (M5-03 · M5-07 · M5-13 · M5-17) đều có chỗ LỌT ở bộ DÀN DỰNG.</t>
+        </is>
+      </c>
+      <c r="W106" s="26" t="inlineStr">
+        <is>
+          <t>4 lần nén C2 ĐẠT trên sổ cái thật, 0 lần huỷ, ở 2 dự án (robot-tu-can-bang, thu-nghiem-mem-c) — và bản tóm tắt cuối nạp lại được qua tu_dict, KHÔNG rỗng, ở 2/2. 313 phiên có transcript, 303 (96 %) thuộc dự án CHƯA TỪNG NÉN: câu 'chưa có bản tóm tắt nào' là câu khối resume nói ở gần như mọi lần mở lại, trong khi một transcript đầy đủ đang nằm sẵn trên đĩa. LỖI TRONG CHÍNH PHÉP ĐO: phép đếm đầu tiên lọc bằng '"buoc": "ok"' in line, mà sổ cái thật ghi JSON KHÔNG có khoảng trắng sau dấu hai chấm — nên nó trả 100 % thay vì trả rỗng. Cứu được vì grep -c '"compact"' ra 146 dòng, chỏi với kết luận 'chưa nén lần nào'.</t>
+        </is>
+      </c>
+      <c r="X106" s="26" t="inlineStr">
+        <is>
+          <t>RESUME_TUONG_THUAT — mặc định TẮT (phần nạp lại tóm tắt C2 KHÔNG sau cờ)</t>
+        </is>
+      </c>
+      <c r="Y106" s="26" t="inlineStr">
+        <is>
+          <t>Không còn nợ tiêu chí nào. Cờ thứ 12, giữ TẮT. Phần A (nạp lại tóm tắt từ sổ cái) là sửa lỗi thuần nên chạy cả khi cờ tắt. Bỏ phần 'trạng thái kế hoạch vào resume' theo đúng ghi chú của kế hoạch — plan:current đã hiện ở &lt;pending&gt; mỗi lượt.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="102" customHeight="1" s="27">
       <c r="A107" s="46" t="inlineStr">

</xml_diff>

<commit_message>
Cất việc #24 → #32: README, DANG-LAM và sheet tiến độ mới
30/106 việc xong, và HẾT P0 KHÔNG BỊ CHẶN của Giai đoạn 1 (GĐ1 có 32 việc; còn #26
M2-09 là P1 · L và #27 M4-13 bị nó chặn). Bộ kiểm 1 610 → 2 030 · 12 cờ · 132 công cụ ·
DEV-330 → DEV-359.

README: năm dòng mới vào bảng đợt rà lại, §8 cập nhật mười hai cờ còn TẮT, và nói rõ hai
việc mới nhất KHÔNG đạt 100 % phá-lại-thì-đỏ cùng lý do.

DANG-LAM: viết lại quanh bài học lặp BỐN lần liền của đợt này — chỗ LỌT nằm ở bộ DÀN DỰNG
của ca kiểm, không ở mã sản phẩm (hai vế tình cờ bằng nhau · một tập hợp tình cờ có một
phần tử · một hình dạng tình cờ đã đúng · ca kiểm không chạy tới dòng nó nói nó canh).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
+++ b/toi-uu/EIDE_Toi_uu_Agent_2026-10-06.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu 18 mẫu" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Điểm mạnh cần giữ" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương pháp &amp; nguồn" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ 09-10-2026 (sau #32)" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Danh mục tối ưu'!$A$4:$S$110</definedName>
@@ -2105,17 +2106,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B51:G51"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="A41:G41"/>
     <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="A45:G45"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3868,7 +3869,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="27">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -15748,6 +15748,1962 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" style="27" min="1" max="1"/>
+    <col width="66" customWidth="1" style="27" min="2" max="2"/>
+    <col width="24" customWidth="1" style="27" min="3" max="3"/>
+    <col width="8" customWidth="1" style="27" min="4" max="4"/>
+    <col width="11" customWidth="1" style="27" min="5" max="5"/>
+    <col width="16" customWidth="1" style="27" min="6" max="6"/>
+    <col width="34" customWidth="1" style="27" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>TIẾN ĐỘ ĐỢT TỐI ƯU TÁC TỬ — chốt sau việc #32, 09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Mỗi dòng 'Xong' đều có: mục DEV-LOG tra lại được · số ca kiểm trước→sau · một con số đo trên dữ liệu thật · phần còn nợ. Cột chi tiết nằm ở sheet “Danh mục tối ưu”, cột T–Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Tổng quan</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Số việc</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Xong (đã gộp vào main, đã đẩy)</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>30/106 — và HẾT P0 KHÔNG BỊ CHẶN của Giai đoạn 1. GĐ1 có 32 việc; còn #26 M2-09 (P1 · L, tiền đề cứng) và #27 M4-13 (P0 · M, bị #26 chặn).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Đang làm (chưa commit)</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>không việc nào đang dở; main đã đẩy và khớp origin/main</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="n">
+        <v>76</v>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>76 việc còn lại trong 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="n">
+        <v>106</v>
+      </c>
+      <c r="C8" s="61" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>Phép đo của cả đợt</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>Trước (06/10)</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Sau (09/10 sau #32)</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị Python (pytest -q)</t>
+        </is>
+      </c>
+      <c r="B11" s="63" t="inlineStr">
+        <is>
+          <t>1 610</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>2 030</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>+420 ca so với 06/10; 1 skip (cần tệp .svd thật, máy không có); không ca cũ nào đỏ ở bất kỳ bước nào</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>Ca đơn vị giao diện (swift test)</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>không nhiệm vụ nào đụng ui/ — kiểu khối A2.2 dùng “table”, Swift đã dựng được</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="63" t="inlineStr">
+        <is>
+          <t>kiem_tai_lieu.py</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ lệch</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>0 chỗ LỆCH CHẮC CHẮN mọi lượt. M4-07 không thêm công cụ nào, nên số công cụ giữ 131 — nhưng nó SỬA chỗ đếm: kiem_tai_lieu bật mọi cờ theo Features.ten_co(), và danh sách ấy gõ tay nên cờ thứ 10 vô hình với nó</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>thu_sch.py (cờ schematic bật)</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>63/63</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>chạy ở M3-03 và M3-04, không tụt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Mục DEV-LOG mới</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330 → DEV-359</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>30 mục, mỗi việc một mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>Cờ tính năng mới</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>1 (schematic)</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>11 cờ mới, TẤT CẢ mặc định TẮT. Hai cờ mới nhất: HOI_QUY_NEN (M4-11) và RESUME_TUONG_THUAT (M5-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>Mã lỗi mới</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>E4031 · E4032 · E6012 · E4033 · E4024 · E2007 · E2008</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>M5-03 dùng E2007 (SVD không đọc được); M5-07 dùng E2008 cho BA lý do mới và GIỮ E2006 cho 'giá trị không có trong đoạn' — bốn lý do dẫn tới bốn việc khác nhau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>Mảng</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>Ưu tiên</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>DEV-LOG</t>
+        </is>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Ca kiểm</t>
+        </is>
+      </c>
+      <c r="G19" s="59" t="inlineStr">
+        <is>
+          <t>Cờ mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>M1-01</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="inlineStr">
+        <is>
+          <t>DEV-330</t>
+        </is>
+      </c>
+      <c r="F20" s="63" t="inlineStr">
+        <is>
+          <t>105/309 phiên thật có lịch sử tự mâu thuẫn — 255 chỗ (156 kết quả thứ hai cùng id, 74 message chen giữa, 24 kết quả lạc lượt, 1 lời gọi không kết quả)</t>
+        </is>
+      </c>
+      <c r="G20" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>M1-02</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>DEV-331</t>
+        </is>
+      </c>
+      <c r="F21" s="63" t="inlineStr">
+        <is>
+          <t>lược đồ công cụ thật: 25 869 token/lời gọi (trần tool_schema=4000 chưa dòng mã nào đọc). Cờ bật: 4 475 token, giảm 82,7 %; 73 → 18 công cụ</t>
+        </is>
+      </c>
+      <c r="G21" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>M1-03</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="inlineStr">
+        <is>
+          <t>1. Lõi tác tử</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
+        <is>
+          <t>DEV-332</t>
+        </is>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>1 822 lời gọi của tác tử con trong 26 phiên thật, 0 lần qua lớp luật. Toàn công cụ đọc trừ một build.compile — lỗ hổng chưa bị bước vào, không phải được canh</t>
+        </is>
+      </c>
+      <c r="G22" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>M2-01</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>DEV-333</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>kịch bản 3 REQ + 3 phương án + 3 tiêu chí + 3 tệp: sửa MỘT REQ làm 9 hiện vật STALE → còn 3. Phép đo đầu ra 6→2 vì bị hàng rào E4020 chặn, đã sửa kịch bản đo</t>
+        </is>
+      </c>
+      <c r="G23" s="63" t="inlineStr">
+        <is>
+          <t>TRUY_VET — TẮT (phần nền chạy cả khi tắt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>M2-02</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E24" s="63" t="inlineStr">
+        <is>
+          <t>DEV-334</t>
+        </is>
+      </c>
+      <c r="F24" s="63" t="inlineStr">
+        <is>
+          <t>63 kho thật: 5/37 REQ có ít nhất một phép đo; 27 chưa có phương án nào nhận; 0 REQ đi hết chuỗi. Cột 'Mã nguồn' trống ở MỌI dự án vì hien_thuc_req vừa mới tồn tại</t>
+        </is>
+      </c>
+      <c r="G24" s="63" t="inlineStr">
+        <is>
+          <t>REQ_PHU — TẮT (khối A2.2 trên tab không phụ thuộc cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>M2-03</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E25" s="63" t="inlineStr">
+        <is>
+          <t>DEV-335</t>
+        </is>
+      </c>
+      <c r="F25" s="63" t="inlineStr">
+        <is>
+          <t>37 REQ thật: 25 sạch (67 %), 11 thiếu tiêu chí đo được, 2 có từ mơ hồ. Lần đo đầu ra 3 từ mơ hồ, một là kêu oan ('ít nhất 2 lần' là mức đo được) — đã vá</t>
+        </is>
+      </c>
+      <c r="G25" s="63" t="inlineStr">
+        <is>
+          <t>REQ_CHAT_LUONG — TẮT (module yeu_cau.py luôn có)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>M2-06</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="inlineStr">
+        <is>
+          <t>DEV-336</t>
+        </is>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>sổ cái thật: 26 lần đánh dấu 'xong' ngay sau một lần ghi mã, 19 lần (73 %) không có phép kiểm nào đạt ở giữa. Phép đo đầu ở mức dự án ra 0 — đúng nhưng đo sai câu hỏi</t>
+        </is>
+      </c>
+      <c r="G26" s="63" t="inlineStr">
+        <is>
+          <t>KE_HOACH_CONG_KIEM — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>M2-08</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>2. Phân tích &amp; thiết kế phần mềm</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="inlineStr">
+        <is>
+          <t>DEV-337</t>
+        </is>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>185 tệp .c thật: 1 758 → 1 786 hàm thấy được (+28 hàm trước đây VÔ HÌNH: 8 ngắt + 20 bị regex tham lam nuốt). 78 hàm nay gắn nhãn 'isr', 70 trong đó vốn đã có trong danh sách</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>DEV-338</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mô hình mạch thật — và lý do đáng hơn con số: 3 kho CÓ Fact v_max thì KHÔNG có mô hình mạch, 5 kho có mạch thì không có Fact ấy; thêm nữa Fact dùng chủ thể chip:X mà ERC không tra tiền tố đó</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E29" s="63" t="inlineStr">
+        <is>
+          <t>DEV-339</t>
+        </is>
+      </c>
+      <c r="F29" s="63" t="inlineStr">
+        <is>
+          <t>8 phát hiện trên 5 mạch thật (6 nguon_khong_cap + 2 net_mot_chan), trong đó net clock I2C nối đúng một chân. SÁU trong tám là 'mô hình chưa khai' chứ không phải 'mạch sai'. robot-canbang: 107 Port lá, KHÔNG Port nào là power_out</t>
+        </is>
+      </c>
+      <c r="G29" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E30" s="63" t="inlineStr">
+        <is>
+          <t>DEV-340</t>
+        </is>
+      </c>
+      <c r="F30" s="63" t="inlineStr">
+        <is>
+          <t>0 phát hiện trên 5 mạch thật — và đây là con số ĐÚNG (hai lỗi này catastrophic, không bo nào sống tới lúc lưu kho). Đã CẤY hai bộ cấp vào bản sao kho robot-canbang để chứng minh luật sống: nổ đúng 1 blocker trên net +5V thật</t>
+        </is>
+      </c>
+      <c r="G30" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>M3-07</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E31" s="63" t="inlineStr">
+        <is>
+          <t>DEV-341</t>
+        </is>
+      </c>
+      <c r="F31" s="63" t="inlineStr">
+        <is>
+          <t>Fact tới được ERC: 5 → 17 (+12). Ba kho có Fact datasheet thì TOÀN BỘ mang chủ thể chip:, tức trước đó không một Fact nào tới được ERC. Độ phủ 5 mạch thật nay đọc được</t>
+        </is>
+      </c>
+      <c r="G31" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>M3-10</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E32" s="63" t="inlineStr">
+        <is>
+          <t>DEV-342</t>
+        </is>
+      </c>
+      <c r="F32" s="63" t="inlineStr">
+        <is>
+          <t>chi phí đo thật: mạch lớn nhất trong kho 187 nút → ERC 7,6 ms mỗi lần ghi. Trần 2000 nút, vượt thì NÓI RA chứ không im lặng bỏ qua</t>
+        </is>
+      </c>
+      <c r="G32" s="63" t="inlineStr">
+        <is>
+          <t>ERC_TU_DONG — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>M3-12</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E33" s="63" t="inlineStr">
+        <is>
+          <t>DEV-343</t>
+        </is>
+      </c>
+      <c r="F33" s="63" t="inlineStr">
+        <is>
+          <t>846 bản ghi mô phỏng thật: regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 (testbench dự án in 'KET QUA: PASS' — nhãn đứng TRƯỚC từ khoá). Nới đúng một chỗ → 846/846 khớp, vẫn bắt đủ bốn ca PASS giả</t>
+        </is>
+      </c>
+      <c r="G33" s="63" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="64" t="inlineStr">
+        <is>
+          <t>M3-13</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="inlineStr">
+        <is>
+          <t>DEV-344</t>
+        </is>
+      </c>
+      <c r="F34" s="64" t="inlineStr">
+        <is>
+          <t>testbench Verilog THẬT của bài 3: tb_pcpi_dot4 1/1, tb_pcpi_mac 1/1, tb_pcpi_vmini không đo được (tb gọi bản bram HAI CỔNG đã bị bỏ 02/10) — mẫu số là TỆP, không phải phép phá</t>
+        </is>
+      </c>
+      <c r="G34" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>M3-18</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>3. Mạch, ERC, HDL/FPGA</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="inlineStr">
+        <is>
+          <t>DEV-345</t>
+        </is>
+      </c>
+      <c r="F35" s="64" t="inlineStr">
+        <is>
+          <t>6 cặp (mạng cổng, .cst) thật → 1 chỗ CHẶN: blinky của riscv-tn20k-b dựng bitstream 4,6 MB với chân đồng hồ do nextpnr tự chọn (rơi đúng chân 4 — bằng may). Cả 7 tệp .cst thật đọc hết, 0 lỗi cú pháp</t>
+        </is>
+      </c>
+      <c r="G35" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B36" s="64" t="inlineStr">
+        <is>
+          <t>M4-01</t>
+        </is>
+      </c>
+      <c r="C36" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D36" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E36" s="64" t="inlineStr">
+        <is>
+          <t>DEV-346</t>
+        </is>
+      </c>
+      <c r="F36" s="64" t="inlineStr">
+        <is>
+          <t>18 ca chạy trình biên dịch C thật: tệp test in số đo {"T1":300} với ngưỡng &lt;=255 → EIDE phán 1 ca HỎNG. Chưa kho cũ nào có tiêu chí unit test để đo lại trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="G36" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (công cụ mới core=False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B37" s="64" t="inlineStr">
+        <is>
+          <t>M4-02</t>
+        </is>
+      </c>
+      <c r="C37" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D37" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E37" s="64" t="inlineStr">
+        <is>
+          <t>DEV-347</t>
+        </is>
+      </c>
+      <c r="F37" s="64" t="inlineStr">
+        <is>
+          <t>25 ca dựng đúng trạng thái thật (tệp test 3 ca, 1 ca đỏ, hiện vật dat=False) → fs.write còn 1 ca thì test.weakened=True. Và hàng rào cũ criteria.has_result chưa bao giờ nổ ngoài sim-01</t>
+        </is>
+      </c>
+      <c r="G37" s="64" t="inlineStr">
+        <is>
+          <t>SIM_RUNNER_GIOI_HAN — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="64" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B38" s="64" t="inlineStr">
+        <is>
+          <t>M4-05</t>
+        </is>
+      </c>
+      <c r="C38" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D38" s="64" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E38" s="64" t="inlineStr">
+        <is>
+          <t>DEV-348</t>
+        </is>
+      </c>
+      <c r="F38" s="64" t="inlineStr">
+        <is>
+          <t>du-lieu/rtos-sinhvien, chạy CẢ HAI hành vi: cũ so_thay=1, mới so_thay=0 — logo_ptit.c từ 'bộ kiểm ĐỎ' thành 'mọi đột biến đều làm hỏng biên dịch'. Một ô xanh giả, đã sửa</t>
+        </is>
+      </c>
+      <c r="G38" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="64" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B39" s="64" t="inlineStr">
+        <is>
+          <t>M4-19</t>
+        </is>
+      </c>
+      <c r="C39" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D39" s="64" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E39" s="64" t="inlineStr">
+        <is>
+          <t>DEV-349</t>
+        </is>
+      </c>
+      <c r="F39" s="64" t="inlineStr">
+        <is>
+          <t>chạy TẠI CHỖ trên ba dự án firmware thật: kết luận giống hệt lượt đột biến tại chỗ của M4-05, và 50/50 tệp giữ nguyên cả sha256 lẫn mtime</t>
+        </is>
+      </c>
+      <c r="G39" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="64" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B40" s="64" t="inlineStr">
+        <is>
+          <t>M4-04</t>
+        </is>
+      </c>
+      <c r="C40" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D40" s="64" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E40" s="64" t="inlineStr">
+        <is>
+          <t>DEV-350</t>
+        </is>
+      </c>
+      <c r="F40" s="64" t="inlineStr">
+        <is>
+          <t>TÁI HIỆN được ca DANH-GIA §2.2 bằng máy trên control_rtos.c thật: bảng cũ 0 đột biến cho hằng hex, bảng mới dòng 147 → mutant SỐNG. Và chi_tiet trên 12 tệp thật: 110 s, điểm 0,0</t>
+        </is>
+      </c>
+      <c r="G40" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ (tham số mới, mặc định giữ hành vi cũ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="64" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B41" s="64" t="inlineStr">
+        <is>
+          <t>M4-06</t>
+        </is>
+      </c>
+      <c r="C41" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D41" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E41" s="64" t="inlineStr">
+        <is>
+          <t>DEV-351</t>
+        </is>
+      </c>
+      <c r="F41" s="64" t="inlineStr">
+        <is>
+          <t>đo TRƯỚC trên logo_ptit.c thật: điểm 0,0 · 30 mutant · 20 sống. Phần SAU chưa đo — cần lời gọi mô hình (§3.0 bắt hỏi trước), và dự án mẫu không có chỗ để đo</t>
+        </is>
+      </c>
+      <c r="G41" s="64" t="inlineStr">
+        <is>
+          <t>TEST_HARDEN — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="64" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B42" s="64" t="inlineStr">
+        <is>
+          <t>M4-07</t>
+        </is>
+      </c>
+      <c r="C42" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D42" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E42" s="64" t="inlineStr">
+        <is>
+          <t>DEV-352</t>
+        </is>
+      </c>
+      <c r="F42" s="64" t="inlineStr">
+        <is>
+          <t>sổ cái 42 dự án: 327 lời gọi task.run có việc, 323 là verifier · 209/323 đề bài dài hơn trần 300 ký tự · gói bằng chứng dựng được CÓ NỘI DUNG trên 29/42 dự án, 0 lần đổ · loc_claim bỏ 95/1 706 câu (năm dấu hiệu kế hoạch chỉ bỏ được 11)</t>
+        </is>
+      </c>
+      <c r="G42" s="64" t="inlineStr">
+        <is>
+          <t>VERIFIER_GOI_BANG_CHUNG — TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="64" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B43" s="64" t="inlineStr">
+        <is>
+          <t>M4-09</t>
+        </is>
+      </c>
+      <c r="C43" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D43" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E43" s="64" t="inlineStr">
+        <is>
+          <t>DEV-353</t>
+        </is>
+      </c>
+      <c r="F43" s="64" t="inlineStr">
+        <is>
+          <t>68 sổ cái: hook Stop khai tu_kiem_da_chay ở 41 lượt, và 1 trong 41 lượt ấy KHÔNG có task.run(verifier) nào — robot-sinhvien2 run-007, nơi lời gọi làm hook im nằm TRƯỚC fs.edit vào ISR(TIMER2_COMPA_vect). Phá lại thì đỏ 10/12.</t>
+        </is>
+      </c>
+      <c r="G43" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="64" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B44" s="64" t="inlineStr">
+        <is>
+          <t>M4-11</t>
+        </is>
+      </c>
+      <c r="C44" s="64" t="inlineStr">
+        <is>
+          <t>4. Kiểm thử &amp; chất lượng</t>
+        </is>
+      </c>
+      <c r="D44" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E44" s="64" t="inlineStr">
+        <is>
+          <t>DEV-354</t>
+        </is>
+      </c>
+      <c r="F44" s="64" t="inlineStr">
+        <is>
+          <t>9 kho thật: bán kính STALE của kết quả test/sim khi sửa một tệp mã 107 → 49 lần (58/107 là cáo buộc OAN). Dữ liệu thật bác bước 1 của kế hoạch: robot-sinhvien2 lưu MỘT tệp nguồn, mà tệp ấy #include ba tệp firmware. Phá lại thì đỏ 24/32 → 31/34.</t>
+        </is>
+      </c>
+      <c r="G44" s="64" t="inlineStr">
+        <is>
+          <t>HOI_QUY_NEN — TẮT (deps.upstream + hook ket_qua_stale KHÔNG sau cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="64" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B45" s="64" t="inlineStr">
+        <is>
+          <t>M5-03</t>
+        </is>
+      </c>
+      <c r="C45" s="64" t="inlineStr">
+        <is>
+          <t>5. Tri thức &amp; tài liệu</t>
+        </is>
+      </c>
+      <c r="D45" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E45" s="64" t="inlineStr">
+        <is>
+          <t>DEV-355</t>
+        </is>
+      </c>
+      <c r="F45" s="64" t="inlineStr">
+        <is>
+          <t>grep -rni svd src/ TRƯỚC khi sửa ra đúng HAI chỗ: phép phân loại, và một comment nói 'bốn loại đó có công cụ riêng' — không có bộ đọc nào. Tức phan_loai khai ĐẦY ĐỦ còn doc.load trả E1001. Phá lại thì đỏ 28/34 → 34/34.</t>
+        </is>
+      </c>
+      <c r="G45" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần + công cụ mới core=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="64" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B46" s="64" t="inlineStr">
+        <is>
+          <t>M5-05</t>
+        </is>
+      </c>
+      <c r="C46" s="64" t="inlineStr">
+        <is>
+          <t>5. Tri thức &amp; tài liệu</t>
+        </is>
+      </c>
+      <c r="D46" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E46" s="64" t="inlineStr">
+        <is>
+          <t>DEV-356</t>
+        </is>
+      </c>
+      <c r="F46" s="64" t="inlineStr">
+        <is>
+          <t>hop_ly('vdd.max', 25, '°C') trả True trên mã cũ — 25 lọt khoảng điện áp 0,5–60 V. Và đường BẢNG sinh khoá khác đường DÒNG CHỮ (flash.size → flash.max), nên một dung lượng Flash đọc từ bảng chưa bao giờ thành hạn mức. Phá lại thì đỏ 17/21 → 23/24.</t>
+        </is>
+      </c>
+      <c r="G46" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="64" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B47" s="64" t="inlineStr">
+        <is>
+          <t>M5-07</t>
+        </is>
+      </c>
+      <c r="C47" s="64" t="inlineStr">
+        <is>
+          <t>5. Tri thức &amp; tài liệu</t>
+        </is>
+      </c>
+      <c r="D47" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E47" s="64" t="inlineStr">
+        <is>
+          <t>DEV-357</t>
+        </is>
+      </c>
+      <c r="F47" s="64" t="inlineStr">
+        <is>
+          <t>Phép kiểm cũ xoá hết dấu chấm rồi so chuỗi chứa: '2.7 V' thành '27v' nên giá trị '27' đi qua, và '3' khớp 'Table 3', '180' khớp '1800', '39' khớp '0.39'. Phá lại thì đỏ 15/22 → 22/22; cả bảy chỗ LỌT là ca kiểm chưa chạm tới.</t>
+        </is>
+      </c>
+      <c r="G47" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="64" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B48" s="64" t="inlineStr">
+        <is>
+          <t>M5-13</t>
+        </is>
+      </c>
+      <c r="C48" s="64" t="inlineStr">
+        <is>
+          <t>5. Tri thức &amp; tài liệu</t>
+        </is>
+      </c>
+      <c r="D48" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E48" s="64" t="inlineStr">
+        <is>
+          <t>DEV-358</t>
+        </is>
+      </c>
+      <c r="F48" s="64" t="inlineStr">
+        <is>
+          <t>23 kho thật: một lời gọi fact.query không tham số đưa 67 635 → 32 560 token vào ngữ cảnh (−51 %); robot-sinhvien một mình 12 076 → 4 579. Trần chung bị LÁCH vì _cat_chung cắt số phần tử mà không cắt phần tử. Phá lại thì đỏ 20/23 → 23/23.</t>
+        </is>
+      </c>
+      <c r="G48" s="64" t="inlineStr">
+        <is>
+          <t>không có cờ — sửa lỗi thuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="64" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B49" s="64" t="inlineStr">
+        <is>
+          <t>M5-17</t>
+        </is>
+      </c>
+      <c r="C49" s="64" t="inlineStr">
+        <is>
+          <t>5. Tri thức &amp; tài liệu</t>
+        </is>
+      </c>
+      <c r="D49" s="64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E49" s="64" t="inlineStr">
+        <is>
+          <t>DEV-359</t>
+        </is>
+      </c>
+      <c r="F49" s="64" t="inlineStr">
+        <is>
+          <t>4 lần nén C2 đạt trên sổ cái thật (2 dự án), bản tóm tắt nạp lại được và KHÔNG rỗng ở 2/2. Và 303/313 phiên (96 %) thuộc dự án CHƯA TỪNG NÉN — nên câu 'chưa có bản tóm tắt' là câu nói ở gần như mọi lần mở lại. Phá lại thì đỏ 20/23 → 23/23.</t>
+        </is>
+      </c>
+      <c r="G49" s="64" t="inlineStr">
+        <is>
+          <t>RESUME_TUONG_THUAT — TẮT (phần nạp lại tóm tắt C2 KHÔNG sau cờ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="59" t="inlineStr">
+        <is>
+          <t>Việc còn MỞ (ngoài 84 việc chưa làm)</t>
+        </is>
+      </c>
+      <c r="B50" s="59" t="inlineStr">
+        <is>
+          <t>Vì sao còn mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="63" t="inlineStr">
+        <is>
+          <t>Bảy cờ mới đều còn TẮT</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="inlineStr">
+        <is>
+          <t>GON_CONG_CU · TRUY_VET · REQ_PHU · REQ_CHAT_LUONG · KE_HOACH_CONG_KIEM · ERC_TU_DONG · SIM_RUNNER_GIOI_HAN. Cả bảy đổi thứ Agent nhìn thấy, đọc, hoặc LÀM ĐƯỢC mỗi lượt, nên chỉ bộ 76 ca chạy hai chế độ mới nói được chúng làm Agent khá hơn hay tệ hơn. Bộ ấy tốn tiền mô hình nên §3.0 bắt hỏi người dùng trước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="63" t="inlineStr">
+        <is>
+          <t>kiem_cap_goi_tra() chưa thành hàng rào</t>
+        </is>
+      </c>
+      <c r="B52" s="63" t="inlineStr">
+        <is>
+          <t>Soát được mọi phiên đã lưu, nhưng chưa hook nào gọi nó tự động — bắt được chuyện cũ, chưa chặn được chuyện mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="63" t="inlineStr">
+        <is>
+          <t>Luật ERC quá áp chưa nổ trên dữ liệu thật</t>
+        </is>
+      </c>
+      <c r="B53" s="63" t="inlineStr">
+        <is>
+          <t>Đường dẫn đã thông ở M3-07, nhưng ba kho có Fact điện áp thì không có mô hình mạch, và ngược lại. Phải chờ một dự án có cả hai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="63" t="inlineStr">
+        <is>
+          <t>Cột “Mã nguồn” của ma trận truy vết trống ở mọi dự án</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="inlineStr">
+        <is>
+          <t>Nó đọc hien_thuc_req — trường vừa mới tồn tại, chưa tệp nào trên đĩa từng khai. Nên “chưa hiện thực” ở đó nghĩa là “chưa ai KHAI”, không phải “chưa ai viết”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="63" t="inlineStr">
+        <is>
+          <t>Lỗi _go_dau trong src/eide/tools/design.py</t>
+        </is>
+      </c>
+      <c r="B55" s="63" t="inlineStr">
+        <is>
+          <t>Viết .replace('d','d') nên 'ổn định' và 'ON DINH' không khớp nhau. Hàm ấy đang dùng cho một phép kiểm an toàn (người có thật sự chọn không). Tìm thấy ở M2-03, CHƯA sửa vì ngoài phạm vi — cần bộ ca kiểm riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="63" t="inlineStr">
+        <is>
+          <t>subagent req-critic (bước 4 của M2-03)</t>
+        </is>
+      </c>
+      <c r="B56" s="63" t="inlineStr">
+        <is>
+          <t>Kế hoạch ghi “tuỳ chọn, gộp M2-13”. Chưa làm, đúng theo kế hoạch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="63" t="inlineStr">
+        <is>
+          <t>Hai luật kiểm chân FPGA chưa có dữ liệu để nổ</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="inlineStr">
+        <is>
+          <t>chan_lech_kit và io_type_lech_bank cần Fact chân kit. Không kho nào trong repo có Fact pin:tangnano20k.* hay khoá vccio — nên hôm nay chỉ 3 trong 5 luật của M3-18 kết luận được gì trên dữ liệu thật. Cùng hình dạng với luật ERC quá áp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="63" t="inlineStr">
+        <is>
+          <t>Một bitstream cũ đã dựng với chân đồng hồ tự chọn</t>
+        </is>
+      </c>
+      <c r="B58" s="63" t="inlineStr">
+        <is>
+          <t>blinky của du-lieu/riscv-tn20k-b — xem DEV-345 và README §8. Không sửa hiện vật cũ: đó là dữ liệu của những lượt đo đã chốt. Từ nay phép kiểm chặn trước nextpnr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="63" t="inlineStr">
+        <is>
+          <t>Ba công cụ mới nhất chưa lượt Agent nào GỌI</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="inlineStr">
+        <is>
+          <t>hdl.sensitivity · hdl.constraints_check · test.criteria. Mã của cả ba đã chạy trên hiện vật thật, nhưng đó là tôi gọi hàm, không phải tác tử gọi công cụ. README §8 đếm cả ba vào phần chưa dùng thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="63" t="inlineStr">
+        <is>
+          <t>Bộ kiểm C của ba dự án firmware thật đều KHÔNG đo được độ nhạy</t>
+        </is>
+      </c>
+      <c r="B60" s="63" t="inlineStr">
+        <is>
+          <t>rtos-sinhvien: 0/12 tệp đo được (4 font khong_thay, control_rtos.c trùng ký hiệu, main.c không dịch trên máy chủ, logo_ptit.c mọi mutant hỏng biên dịch). stm32f469-freertos và thu-nghiem-g6: bộ kiểm ĐỎ SẴN. Đây là trạng thái của dữ liệu đo, không phải lỗi sản phẩm — nhưng nó nghĩa là chưa dự án firmware nào trong repo có một con số độ nhạy đáng tin. Xem DEV-348.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="63" t="inlineStr">
+        <is>
+          <t>POL-N6-sua-test chưa nổ trên một phiên thật nào</t>
+        </is>
+      </c>
+      <c r="B61" s="63" t="inlineStr">
+        <is>
+          <t>Hook sua_test_sau_do cấp dữ kiện cho lời gọi SẮP xảy ra, nên không soát lại được phiên đã lưu — khác mọi phép đo trước của đợt này. Nó đã có 25 ca kiểm và phá lại 27/27, nhưng chưa lượt tác tử thật nào chạm vào nó. Cùng hình dạng với ba luật kiểm thiếu dữ liệu ở trên, chỉ khác lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="63" t="inlineStr">
+        <is>
+          <t>Tiêu chí 'mutation score tăng sau harden' của M4-06 chưa đo</t>
+        </is>
+      </c>
+      <c r="B62" s="63" t="inlineStr">
+        <is>
+          <t>Cần LỜI GỌI MÔ HÌNH, và §3.0 bắt hỏi anh Công trước. Đo 'trước' đã có (điểm 0,0 trên logo_ptit.c). Và dự án mẫu không có chỗ để đo: control_rtos.c là khong_nap_duoc, sáu tệp còn lại là bitmap. Cờ TEST_HARDEN giữ TẮT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="63" t="inlineStr">
+        <is>
+          <t>Một dự án chỉ dùng được MỘT tệp test</t>
+        </is>
+      </c>
+      <c r="B63" s="63" t="inlineStr">
+        <is>
+          <t>chay_test dịch MỌI tệp trong test/ cùng nhau, nên tệp thứ hai có main() là trùng ký hiệu. Kiểm trên dữ liệu thật: cả bốn dự án có test/ đều đúng một tệp. M4-06 lách bằng cách thêm ca vào tệp đang có — nhưng ràng buộc ấy vẫn còn, và nó giới hạn cách tổ chức bộ kiểm của mọi dự án.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="63" t="inlineStr">
+        <is>
+          <t>Gói bằng chứng chưa lần nào tới một MÔ HÌNH thật</t>
+        </is>
+      </c>
+      <c r="B64" s="63" t="inlineStr">
+        <is>
+          <t>Nó dựng được trên 29/42 dự án và đọc rất rõ với người, nhưng 'verifier đọc gói này có bác đúng hơn không' là câu hỏi về HÀNH VI MÔ HÌNH, và nó chưa được đo. Tiêu chí xong của M4-07 đòi bộ ca gài lỗi M4-22 — mà M4-22 nằm ở nhiệm vụ SAU trong kế hoạch. Cờ VERIFIER_GOI_BANG_CHUNG giữ TẮT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="63" t="inlineStr">
+        <is>
+          <t>loc_claim là một phép lọc văn xuôi, và nó leaky CÓ SỐ ĐO</t>
+        </is>
+      </c>
+      <c r="B65" s="63" t="inlineStr">
+        <is>
+          <t>95 trong 1 706 câu của 323 đề bài thật. Một câu lập luận không mang chữ nào trong sáu dấu hiệu vẫn đi qua. Đừng nhầm nó với hàng rào — hàng rào là gói bằng chứng do MÃ dựng, thứ tác tử chính không soạn được.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="59" t="inlineStr">
+        <is>
+          <t>Lỗi tìm thấy trong CHÍNH PHÉP ĐO của tôi</t>
+        </is>
+      </c>
+      <c r="B66" s="59" t="inlineStr">
+        <is>
+          <t>Lộ ra ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="63" t="inlineStr">
+        <is>
+          <t>Kịch bản đo bị hàng rào của sản phẩm chặn (ghi tệp chưa đọc, E4020) và trả về một con số hợp lý thay vì nổ — 6→2 trông đẹp y như 9→3 đúng</t>
+        </is>
+      </c>
+      <c r="B67" s="63" t="inlineStr">
+        <is>
+          <t>M2-01 · DEV-333</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm dựng trên điều tôi tự nhớ sai: “thiết” bỏ dấu KHÔNG chứa “it”; chỗ va thật là bit/unit/init/exit</t>
+        </is>
+      </c>
+      <c r="B68" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá dài ĐÚNG BẰNG mã gốc (0.6 → 0.0) nên __pycache__ cũ còn hiệu lực — phép đo chạy mã khác với mã trong tệp</t>
+        </is>
+      </c>
+      <c r="B69" s="63" t="inlineStr">
+        <is>
+          <t>M2-03 · DEV-335</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="63" t="inlineStr">
+        <is>
+          <t>Phép đo trả lời ĐÚNG một câu hỏi KHÁC: đếm ở mức dự án ra 0 chỗ cần chặn; câu phải hỏi là “lần ghi NÀY đã được kiểm chưa” → 19/26</t>
+        </is>
+      </c>
+      <c r="B70" s="63" t="inlineStr">
+        <is>
+          <t>M2-06 · DEV-336</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm RỖNG: dàn dựng không có net đất nào, nên nó xanh cả khi tôi bỏ hẳn phép bỏ qua net đất</t>
+        </is>
+      </c>
+      <c r="B71" s="63" t="inlineStr">
+        <is>
+          <t>M3-01 · DEV-338</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="63" t="inlineStr">
+        <is>
+          <t>Hai phép phá chỉ ra THIẾT KẾ sai, không chỉ ca kiểm yếu (miễn net đất quá rộng; nhánh iout_max chưa ca nào chạm tới)</t>
+        </is>
+      </c>
+      <c r="B72" s="63" t="inlineStr">
+        <is>
+          <t>M3-03 · DEV-339</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="63" t="inlineStr">
+        <is>
+          <t>Phép phá của tôi cũng SAI, và ca âm xanh vì lý do khác — hai cái sai che nhau</t>
+        </is>
+      </c>
+      <c r="B73" s="63" t="inlineStr">
+        <is>
+          <t>M3-07 · DEV-341</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm đo chính câu lệnh của mình (đặt bộ đếm = 3 rồi khẳng định nó khác rỗng, trong khi thực tế nó rỗng)</t>
+        </is>
+      </c>
+      <c r="B74" s="63" t="inlineStr">
+        <is>
+          <t>M3-10 · DEV-342</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="63" t="inlineStr">
+        <is>
+          <t>Regex mà KẾ HOẠCH ghi sẵn từ chối oan 588/846 bản ghi thật; và ba ca kiểm xanh vì lý do sai (tệp giả dùng $4 thay $3; “FAILED” chứa “FAIL”)</t>
+        </is>
+      </c>
+      <c r="B75" s="63" t="inlineStr">
+        <is>
+          <t>M3-12 · DEV-343</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="63" t="inlineStr">
+        <is>
+          <t>"Phá lại thì đỏ 6/6" sai về TẬP, không sai về số: sáu phép phá ấy chọn đúng sáu chỗ đã có ca canh. Phá bằng tập rộng hơn ra 7/9.</t>
+        </is>
+      </c>
+      <c r="B76" s="63" t="inlineStr">
+        <is>
+          <t>M3-13 · DEV-344</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="63" t="inlineStr">
+        <is>
+          <t>409 'blocker' gần như toàn bộ từ một cặp vô nghĩa (mạng cổng của lõi CPU tổng hợp riêng, không bao giờ đem đặt-đi dây). Con số thật là 1.</t>
+        </is>
+      </c>
+      <c r="B77" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="63" t="inlineStr">
+        <is>
+          <t>Phép quét tệp .cst thật chỉ thu 4 trong 7 tệp mà ca kiểm vẫn xanh — câu 'mọi tệp .cst thật đều đọc được' nói về phần phép quét chạm tới.</t>
+        </is>
+      </c>
+      <c r="B78" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="63" t="inlineStr">
+        <is>
+          <t>Một ca kiểm và một phép phá nhắm hai NHÁNH khác nhau, nên ca mới xanh mà phép phá vẫn LỌT. Mất một lượt mới thấy.</t>
+        </is>
+      </c>
+      <c r="B79" s="63" t="inlineStr">
+        <is>
+          <t>M3-18 · DEV-345</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="63" t="inlineStr">
+        <is>
+          <t>Ca kiểm xanh nhờ một DÒNG KHÁC: kiểm `"TỰ KHAI" in str(kh)` cả khối nên vẫn xanh khi phá chữ ấy ở dòng Kết luận — summary cũng chứa nó. Phép phá bắt được, ca kiểm thì không.</t>
+        </is>
+      </c>
+      <c r="B80" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="63" t="inlineStr">
+        <is>
+          <t>Một phép phá VÔ HIỆU: `them = [] or [[…]]` không đổi hành vi, nên nó báo LỌT oan và suýt làm tôi viết ca kiểm cho một chỗ vốn đã được canh.</t>
+        </is>
+      </c>
+      <c r="B81" s="63" t="inlineStr">
+        <is>
+          <t>M4-01 · DEV-346</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="63" t="inlineStr">
+        <is>
+          <t>HAI phép phá liền nhau VÔ HIỆU ở cùng một dòng: `cu = cu or ""` không đổi hành vi, rồi bỏ is_file() cũng không vì except OSError bắt FileNotFoundError. Phải bỏ cả hai lớp phòng mới phá được.</t>
+        </is>
+      </c>
+      <c r="B82" s="63" t="inlineStr">
+        <is>
+          <t>M4-02 · DEV-347</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="63" t="inlineStr">
+        <is>
+          <t>Một luật mới trỏ tới nhóm dữ kiện chưa khai thì DỪNG CẢ LƯỢT bằng ValueError, không phải 'không nổ' — và nhóm `criteria` của hàng rào N6 cũ cũng chưa bao giờ được khai.</t>
+        </is>
+      </c>
+      <c r="B83" s="63" t="inlineStr">
+        <is>
+          <t>M4-02 · DEV-347</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="63" t="inlineStr">
+        <is>
+          <t>Phép đo ĐỔ ngay lượt đầu trên dữ liệu thật (IndexError), và lỗi ấy nghĩa là test.sensitivity chưa bao giờ chạy nổi trên một tệp firmware thật — mọi con số cũ đều từ tệp nhỏ do ca kiểm tự dựng.</t>
+        </is>
+      </c>
+      <c r="B84" s="63" t="inlineStr">
+        <is>
+          <t>M4-05 · DEV-348</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="63" t="inlineStr">
+        <is>
+          <t>Bốn chỗ LỌT cùng một hình dạng: luật ĐÚNG, nằm ở chỗ ca kiểm không với tới — hai closure, một bảng phép không dựng nổi ca, và một tầng báo lại mà mọi ca cũ đều đi qua với stillborn == 0.</t>
+        </is>
+      </c>
+      <c r="B85" s="63" t="inlineStr">
+        <is>
+          <t>M4-05 · DEV-348</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
+          <t>Tôi thêm MỘT cờ biên dịch để tránh một cáo buộc sai, và nó sinh ra MƯỜI MỘT cáo buộc sai khác: -I che header hệ thống, nên 11/12 tệp bị xếp là 'không dịch được trên máy chủ'. Phải là -iquote.</t>
+        </is>
+      </c>
+      <c r="B86" s="26" t="inlineStr">
+        <is>
+          <t>M4-19 · DEV-349</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
+          <t>Gắn cờ biên dịch cho cả LƯỢT MỐC là đổi chính cái mốc mà mọi so sánh dựa vào — mốc của cả ba dự án thật từ XANH thành ĐỎ.</t>
+        </is>
+      </c>
+      <c r="B87" s="26" t="inlineStr">
+        <is>
+          <t>M4-19 · DEV-349</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="26" t="inlineStr">
+        <is>
+          <t>Phép đo mới TREO 10 phút trên tệp thật đầu tiên — không đổ, không báo gì, nên nó trông như một lượt chạy lâu. liet_ke dựng CẢ TỆP cho MỖI chỗ khớp: 57 600 chỗ × 720 KB ≈ 41 GB việc chuỗi.</t>
+        </is>
+      </c>
+      <c r="B88" s="26" t="inlineStr">
+        <is>
+          <t>M4-04 · DEV-350</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="26" t="inlineStr">
+        <is>
+          <t>Ca kiểm chi phí của tôi KHÔNG bắt được bản chậm, vì tệp dựng dùng hằng hex TRẦN — _bo_che trả về ngay khi không có chỗ giữ. Chính CHÚ THÍCH mỗi dòng của tệp thật mới làm mỗi lượt bỏ che thành một lượt regex thật.</t>
+        </is>
+      </c>
+      <c r="B89" s="26" t="inlineStr">
+        <is>
+          <t>M4-04 · DEV-350</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="26" t="inlineStr">
+        <is>
+          <t>Hook so MỐC THỜI GIAN thay vì số phiên bản: updated_at có độ phân giải thô nên hai lần ghi trong cùng một giây BẰNG NHAU, và phép so 'mới hơn' im lặng sai. Ca kiểm đầu tiên của chính hook ấy đỏ ngay.</t>
+        </is>
+      </c>
+      <c r="B90" s="26" t="inlineStr">
+        <is>
+          <t>M4-06 · DEV-351</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="26" t="inlineStr">
+        <is>
+          <t>Tôi quên mở nhánh và commit thẳng lên main. Nội dung đúng, quy trình §3.1 thì không — đã dựng lại con trỏ toi-uu/M4-06 tại đúng commit.</t>
+        </is>
+      </c>
+      <c r="B91" s="26" t="inlineStr">
+        <is>
+          <t>M4-06 · DEV-351</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="26" t="inlineStr">
+        <is>
+          <t>Năm dấu hiệu mà KẾ HOẠCH nêu cho loc_claim chỉ bỏ được 11 trong 1 706 câu của 323 đề bài THẬT — phép lọc đúng đề mà gần như không chạm gì. Chỗ rò thật là PHÁN QUYẾT TRÍCH SẴN ("kết quả 'dat: false'"), và phải thêm một dấu hiệu thứ sáu mới lên 95/1 706.</t>
+        </is>
+      </c>
+      <c r="B92" s="26" t="inlineStr">
+        <is>
+          <t>M4-07 · DEV-352</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="26" t="inlineStr">
+        <is>
+          <t>Hai phép phá LỌT vì ca kiểm xanh nhờ MỘT DÒNG KHÁC: xoá hẳn khối B khỏi gói bằng chứng mà bộ kiểm vẫn xanh, do ca của khối A đã thấy đúng tên tệp ấy qua dòng changeset. Cùng hình dạng DEV-344.</t>
+        </is>
+      </c>
+      <c r="B93" s="26" t="inlineStr">
+        <is>
+          <t>M4-07 · DEV-352</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
+          <t>Ca kiểm CŨ nêu đúng bất biến "mọi cờ phải có trong ten_co()" mà kiểm nó trên MỘT TÊN GÕ SẴN, nên nó xanh suốt trong khi cờ thứ 10 vô hình: Features.load() trả False cả khi biến môi trường đã đặt. Phép so đúng là so hai TẬP HỢP.</t>
+        </is>
+      </c>
+      <c r="B94" s="26" t="inlineStr">
+        <is>
+          <t>M4-07 · DEV-352</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="26" t="inlineStr">
+        <is>
+          <t>Tôi ghi con số ca kiểm (1 895) vào BỐN tệp tài liệu TRƯỚC khi bộ kiểm đầy đủ chạy xong — số thật là 1 896. Một con số suy ra bằng phép cộng trong đầu trông giống hệt một con số đo được.</t>
+        </is>
+      </c>
+      <c r="B95" s="26" t="inlineStr">
+        <is>
+          <t>M4-07 · DEV-352</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>